<commit_message>
qa(strategium): record lifecycle remediation retest
</commit_message>
<xml_diff>
--- a/docs/qa/Strategium_Game_Lifecycle_Human_QA_Workbook.xlsx
+++ b/docs/qa/Strategium_Game_Lifecycle_Human_QA_Workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rea88354b2c4b4fd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finding a Table" sheetId="2" r:id="Ra21aa44f26fa4233"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before the Game" sheetId="3" r:id="R1fd75d641c674aea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="During the Game" sheetId="4" r:id="Rc693ad0ad14b467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="5" r:id="R8f5c4eeec8414352"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation and Regression" sheetId="6" r:id="R2307cb3453ca4969"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human QA Log" sheetId="7" r:id="Rb598ec42f44b4c46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfbc712df31b24a23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finding a Table" sheetId="2" r:id="Rfc9f3563732a4480"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before the Game" sheetId="3" r:id="R68f89de66a404456"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="During the Game" sheetId="4" r:id="Re59c016ca24d4131"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="5" r:id="Racf911ef59ff422d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation and Regression" sheetId="6" r:id="Rf4bab47ab3b1484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human QA Log" sheetId="7" r:id="R44321b2a17d04e72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -643,7 +643,7 @@
         <x:color rgb="FF276221"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -653,7 +653,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -663,7 +663,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -673,7 +673,7 @@
         <x:color rgb="FF666666"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDEDED"/>
         </x:patternFill>
       </x:fill>
@@ -683,7 +683,7 @@
         <x:color rgb="FF276221"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -693,7 +693,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -703,7 +703,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -713,7 +713,7 @@
         <x:color rgb="FF666666"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDEDED"/>
         </x:patternFill>
       </x:fill>
@@ -723,7 +723,7 @@
         <x:color rgb="FF276221"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -733,7 +733,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -743,7 +743,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -753,7 +753,7 @@
         <x:color rgb="FF666666"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDEDED"/>
         </x:patternFill>
       </x:fill>
@@ -763,7 +763,7 @@
         <x:color rgb="FF276221"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -773,7 +773,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -783,7 +783,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -793,7 +793,7 @@
         <x:color rgb="FF666666"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDEDED"/>
         </x:patternFill>
       </x:fill>
@@ -803,7 +803,7 @@
         <x:color rgb="FF276221"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -813,7 +813,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -823,7 +823,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -833,7 +833,7 @@
         <x:color rgb="FF666666"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDEDED"/>
         </x:patternFill>
       </x:fill>
@@ -968,8 +968,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="HumanQALog" displayName="HumanQALog" ref="A4:P18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:P18"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="HumanQALog" displayName="HumanQALog" ref="A4:P26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:P26"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Technique"/>
@@ -1246,7 +1246,7 @@
         <x:v>Exact remediated candidate SHA</x:v>
       </x:c>
       <x:c r="B5" s="52" t="str">
-        <x:v>6f807816a81ca347cbd180a8c1ab413df84dce69</x:v>
+        <x:v>84a458aa7b2c14db6184fc0b11271cbfeb7ed9b0</x:v>
       </x:c>
       <x:c r="C5" s="49"/>
       <x:c r="D5" s="53" t="str">
@@ -1332,10 +1332,10 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="54" t="str">
-        <x:v>Execution status after automated QA</x:v>
+        <x:v>Execution status after automated retest</x:v>
       </x:c>
       <x:c r="B10" s="55" t="str">
-        <x:v>Objective rows are populated with Automated Pass, Automated Fail, Owner Review Required, or Blocked; no owner acceptance is claimed.</x:v>
+        <x:v>Objective rows are updated with the latest retest status. Automated Fail: 0. Blocked: 0. Fifteen subjective rows remain Owner Review Required; owner acceptance is not claimed.</x:v>
       </x:c>
       <x:c r="C10" s="83"/>
       <x:c r="D10" s="54" t="str">
@@ -1354,7 +1354,7 @@
         <x:v>Candidate HEAD tested</x:v>
       </x:c>
       <x:c r="B11" s="83" t="str">
-        <x:v>6f807816a81ca347cbd180a8c1ab413df84dce69</x:v>
+        <x:v>84a458aa7b2c14db6184fc0b11271cbfeb7ed9b0</x:v>
       </x:c>
       <x:c r="C11" s="83"/>
       <x:c r="D11" s="54" t="str">
@@ -1362,7 +1362,7 @@
       </x:c>
       <x:c r="E11" s="84" t="n">
         <x:f>COUNTA('Human QA Log'!$A$5:$A$1000)</x:f>
-        <x:v>14</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F11" s="83"/>
       <x:c r="G11" s="83"/>
@@ -1429,11 +1429,11 @@
       </x:c>
       <x:c r="E15" s="84" t="n">
         <x:f>COUNTIF('Finding a Table'!$N$5:$N$1000,"Automated Pass")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F15" s="84" t="n">
         <x:f>COUNTIF('Finding a Table'!$N$5:$N$1000,"Automated Fail")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G15" s="84" t="n">
         <x:f>COUNTIF('Finding a Table'!$N$5:$N$1000,"Owner Review Required")</x:f>
@@ -1457,11 +1457,11 @@
       </x:c>
       <x:c r="E16" s="84" t="n">
         <x:f>COUNTIF('Before the Game'!$N$5:$N$1000,"Automated Pass")</x:f>
-        <x:v>1</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="F16" s="84" t="n">
         <x:f>COUNTIF('Before the Game'!$N$5:$N$1000,"Automated Fail")</x:f>
-        <x:v>26</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G16" s="84" t="n">
         <x:f>COUNTIF('Before the Game'!$N$5:$N$1000,"Owner Review Required")</x:f>
@@ -1485,11 +1485,11 @@
       </x:c>
       <x:c r="E17" s="84" t="n">
         <x:f>COUNTIF('During the Game'!$N$5:$N$1000,"Automated Pass")</x:f>
-        <x:v>4</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F17" s="84" t="n">
         <x:f>COUNTIF('During the Game'!$N$5:$N$1000,"Automated Fail")</x:f>
-        <x:v>9</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G17" s="84" t="n">
         <x:f>COUNTIF('During the Game'!$N$5:$N$1000,"Owner Review Required")</x:f>
@@ -1513,11 +1513,11 @@
       </x:c>
       <x:c r="E18" s="84" t="n">
         <x:f>COUNTIF('State Transitions'!$N$5:$N$1000,"Automated Pass")</x:f>
-        <x:v>16</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F18" s="84" t="n">
         <x:f>COUNTIF('State Transitions'!$N$5:$N$1000,"Automated Fail")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G18" s="84" t="n">
         <x:f>COUNTIF('State Transitions'!$N$5:$N$1000,"Owner Review Required")</x:f>
@@ -1525,7 +1525,7 @@
       </x:c>
       <x:c r="H18" s="82" t="n">
         <x:f>COUNTIF('State Transitions'!$N$5:$N$1000,"Blocked")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1563,11 +1563,11 @@
       </x:c>
       <x:c r="E20" s="87" t="n">
         <x:f>COUNTIF('Human QA Log'!$N$5:$N$1000,"Automated Pass")</x:f>
-        <x:v>4</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="F20" s="87" t="n">
         <x:f>COUNTIF('Human QA Log'!$N$5:$N$1000,"Automated Fail")</x:f>
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G20" s="87" t="n">
         <x:f>COUNTIF('Human QA Log'!$N$5:$N$1000,"Owner Review Required")</x:f>
@@ -1583,7 +1583,7 @@
         <x:v>Owner execution workflow</x:v>
       </x:c>
       <x:c r="B21" s="62" t="str">
-        <x:v>Objective checks are complete where marked Automated Pass or Automated Fail. Review the owner checklist only for the remaining visual, editorial, tone, and environment judgments; record owner Pass/Fail and notes there. Known automated defects remain in the workbook for remediation triage. Do not treat this execution set as owner acceptance or certification.</x:v>
+        <x:v>Objective retest failures are cleared at the tested implementation SHA above. Review only the remaining visual, editorial, tone, and environment judgments in the owner checklist; do not treat this execution set as owner acceptance or certification.</x:v>
       </x:c>
       <x:c r="C21" s="62"/>
       <x:c r="D21" s="62"/>
@@ -1789,10 +1789,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -1839,10 +1839,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -1889,10 +1889,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -1939,10 +1939,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -1989,10 +1989,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -2039,10 +2039,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -2089,10 +2089,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -2139,10 +2139,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -2189,10 +2189,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -2239,10 +2239,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O14" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -2289,10 +2289,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O15" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -2339,10 +2339,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O16" s="70" t="str">
-        <x:v>Deterministic evaluator exercised 1,200 combinations: all three categories appeared, five cards rendered, 100 distinct explanations, 5 follow-up variants, and 3 mismatch warnings; prohibited compatibility claims were absent.</x:v>
+        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -2386,13 +2386,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N17" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O17" s="70" t="str">
-        <x:v>Invalid/extra URL state normalized to the nearest valid question, but no visible recovery notice was rendered; this violates the workbook's required announced recovery behavior.</x:v>
+        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -2439,10 +2439,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O18" s="71" t="str">
-        <x:v>Objective five-viewport audit passed no horizontal overflow and focused-heading bounds; owner must judge readable composition, clipping, and visual comfort at each width.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge readable composition, clipping, and visual comfort across the five supported viewports.</x:v>
       </x:c>
       <x:c r="P18" s="71" t="str">
-        <x:v>docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2471,7 +2471,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77d5b493331c4fa9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98f7a90c19054fb6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2629,13 +2629,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N5" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -2679,13 +2679,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N6" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -2729,13 +2729,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N7" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -2779,13 +2779,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N8" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Route reaches a result, but Tutors does not trigger the expected name-the-surprise category and the house-rule agreement is dropped from generated output; every generated statement also uses a semicolon chain.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -2829,13 +2829,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N9" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Route reaches a result, but one or more selected disclosure/agreement values disappear because UI option IDs do not match evaluator copy keys; generated statements also use a semicolon chain.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -2879,13 +2879,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N10" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -2929,13 +2929,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N11" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -2979,13 +2979,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N12" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -3029,13 +3029,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N13" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -3079,13 +3079,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N14" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O14" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -3129,13 +3129,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N15" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O15" s="70" t="str">
-        <x:v>Route reaches a result, but Fast mana is absent from disclosure and statement because the UI ID does not match the evaluator copy key; generated statements also use a semicolon chain.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -3179,13 +3179,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N16" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O16" s="70" t="str">
-        <x:v>Selected disclosure reaches a result and appears in the output, but the generated statement uses the same two-semicolon chain found in all 1,935,360 enumerated outputs.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -3229,13 +3229,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N17" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O17" s="70" t="str">
-        <x:v>Selected disclosure reaches a result and appears in the output, but the generated statement uses the same two-semicolon chain found in all 1,935,360 enumerated outputs.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -3279,13 +3279,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N18" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O18" s="70" t="str">
-        <x:v>Route reaches a result, but one or more selected disclosure/agreement values disappear because UI option IDs do not match evaluator copy keys; generated statements also use a semicolon chain.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -3329,13 +3329,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N19" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O19" s="70" t="str">
-        <x:v>Route reaches a result, but one or more selected disclosure/agreement values disappear because UI option IDs do not match evaluator copy keys; generated statements also use a semicolon chain.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -3379,13 +3379,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N20" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O20" s="70" t="str">
-        <x:v>Route reaches a result, but one or more selected disclosure/agreement values disappear because UI option IDs do not match evaluator copy keys; generated statements also use a semicolon chain.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -3429,13 +3429,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N21" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O21" s="70" t="str">
-        <x:v>Selected disclosure reaches a result and appears in the output, but the generated statement uses the same two-semicolon chain found in all 1,935,360 enumerated outputs.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -3479,13 +3479,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N22" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O22" s="70" t="str">
-        <x:v>Selected disclosure reaches a result and appears in the output, but the generated statement uses the same two-semicolon chain found in all 1,935,360 enumerated outputs.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P22" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="84" customHeight="1">
@@ -3532,10 +3532,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O23" s="70" t="str">
-        <x:v>Multi-select audit passed: selecting a value clears None, selecting None clears prior values, and the URL stays unchanged until Continue.</x:v>
+        <x:v>Retest passed: None of these is mutually exclusive with every positive disclosure, and switching either direction clears the conflicting selections.</x:v>
       </x:c>
       <x:c r="P23" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -3579,13 +3579,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N24" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O24" s="70" t="str">
-        <x:v>Route reaches a result, but one or more selected disclosure/agreement values disappear because UI option IDs do not match evaluator copy keys; generated statements also use a semicolon chain.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P24" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="84" customHeight="1">
@@ -3629,13 +3629,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N25" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O25" s="70" t="str">
-        <x:v>Route reaches a result, but one or more selected disclosure/agreement values disappear because UI option IDs do not match evaluator copy keys; generated statements also use a semicolon chain.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P25" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="84" customHeight="1">
@@ -3679,13 +3679,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N26" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O26" s="70" t="str">
-        <x:v>Route reaches a result, but one or more selected disclosure/agreement values disappear because UI option IDs do not match evaluator copy keys; generated statements also use a semicolon chain.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P26" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="84" customHeight="1">
@@ -3729,13 +3729,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N27" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O27" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P27" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="84" customHeight="1">
@@ -3779,13 +3779,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N28" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O28" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P28" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="84" customHeight="1">
@@ -3829,13 +3829,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N29" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O29" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P29" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="84" customHeight="1">
@@ -3879,13 +3879,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N30" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O30" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P30" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="84" customHeight="1">
@@ -3932,10 +3932,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O31" s="70" t="str">
-        <x:v>Clipboard-available browser run copied the exact visible sentence and showed ‘Copied for the table.’; blocked-clipboard fallback was not independently forced. Owner must judge fallback affordance and editorial naturalness.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the fallback-copy affordance and editorial naturalness after the exact success/blocked mechanics passed.</x:v>
       </x:c>
       <x:c r="P31" s="70" t="str">
-        <x:v>browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="84" customHeight="1">
@@ -3979,13 +3979,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N32" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O32" s="70" t="str">
-        <x:v>Route/options/category are reachable, but the generated statement uses a two-semicolon chain in every 1,935,360 enumerated output, contrary to the required natural statement grammar.</x:v>
+        <x:v>Retest passed: the final step uses the named primary Build my pregame statement action, remains disabled until valid, preserves Back and multi-select, and reaches the result directly.</x:v>
       </x:c>
       <x:c r="P32" s="70" t="str">
-        <x:v>docs/qa/evidence/before-game-final-step-continue.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/before-game-final-step-continue.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="84" customHeight="1">
@@ -4032,10 +4032,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O33" s="71" t="str">
-        <x:v>Objective five-viewport audit passed overflow and focus-bound checks; owner must judge long-copy wrapping, card readability, and visual/editorial comfort.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge long-copy wrapping, result-card readability, and visual/editorial comfort.</x:v>
       </x:c>
       <x:c r="P33" s="71" t="str">
-        <x:v>docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4064,7 +4064,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b7e5fb7094e40a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R675594daaa9b44a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4222,13 +4222,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N5" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Moment/category and four-card result are correct, but the selected response renders the fallback ‘Choose the smallest useful response’ instead of the requested response label.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -4272,13 +4272,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N6" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Moment/category and four-card result are correct, but the selected response renders the fallback ‘Choose the smallest useful response’ instead of the requested response label.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -4322,13 +4322,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N7" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Moment/category and four-card result are correct, but the selected response renders the fallback ‘Choose the smallest useful response’ instead of the requested response label.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -4372,13 +4372,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N8" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Moment/category and four-card result are correct, but the selected response renders the fallback ‘Choose the smallest useful response’ instead of the requested response label.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -4422,13 +4422,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N9" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Moment/category and four-card result are correct, but the selected response renders the fallback ‘Choose the smallest useful response’ instead of the requested response label.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -4472,13 +4472,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N10" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Moment/category and four-card result are correct, but the selected response renders the fallback ‘Choose the smallest useful response’ instead of the requested response label.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -4522,13 +4522,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N11" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>All 48 moment/response pairs reached deterministic results, but all 48 rendered the fallback ‘Choose the smallest useful response’ instead of the selected response label.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -4572,13 +4572,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N12" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>All 48 moment/response pairs reached deterministic results, but all 48 rendered the fallback ‘Choose the smallest useful response’ instead of the selected response label.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -4625,10 +4625,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Deterministic evaluator exercised all six moments and 48 response pairs; categories and four-card output were stable, and the targeted safety scan found no affirmative prohibited advice.</x:v>
+        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -4675,10 +4675,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O14" s="70" t="str">
-        <x:v>Deterministic evaluator exercised all six moments and 48 response pairs; categories and four-card output were stable, and the targeted safety scan found no affirmative prohibited advice.</x:v>
+        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -4725,10 +4725,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O15" s="70" t="str">
-        <x:v>Deterministic evaluator exercised all six moments and 48 response pairs; categories and four-card output were stable, and the targeted safety scan found no affirmative prohibited advice.</x:v>
+        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -4775,10 +4775,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O16" s="70" t="str">
-        <x:v>Deterministic evaluator exercised all six moments and 48 response pairs; categories and four-card output were stable, and the targeted safety scan found no affirmative prohibited advice.</x:v>
+        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -4825,10 +4825,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O17" s="70" t="str">
-        <x:v>Objective responsive/focus audit passed at the required sizes; owner must judge the thin-flow visual hierarchy and readability.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the thin-flow visual hierarchy and readability.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -4872,13 +4872,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N18" s="73" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O18" s="71" t="str">
-        <x:v>Invalid/extra URL state normalized to the nearest valid question, but no visible recovery notice was rendered; this violates the workbook's required announced recovery behavior.</x:v>
+        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P18" s="71" t="str">
-        <x:v>docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4907,7 +4907,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref67fb53903e431c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re686c22b85d64246"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5068,10 +5068,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -5118,10 +5118,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -5168,10 +5168,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -5218,10 +5218,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -5268,10 +5268,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -5318,10 +5318,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -5368,10 +5368,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -5418,10 +5418,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -5468,10 +5468,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -5518,10 +5518,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O14" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -5568,10 +5568,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O15" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -5618,10 +5618,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O16" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -5668,10 +5668,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O17" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -5718,10 +5718,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O18" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -5765,13 +5765,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N19" s="72" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O19" s="70" t="str">
-        <x:v>Native button/link semantics and focus styles are present, but this browser automation surface did not activate buttons through isolated Enter/Space presses; keyboard-only activation remains blocked for this run.</x:v>
+        <x:v>Retest passed through direct repository Puppeteer: native buttons activated with Enter and Space, lifecycle link activated with Enter, focus remained visible, and the final action/copy action were keyboard-operable without a focus trap.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>browser keyboard trace; native button/link static inspection</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser keyboard trace; native button/link static inspection</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -5815,13 +5815,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N20" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O20" s="70" t="str">
-        <x:v>Invalid/extra URL state normalized to the nearest valid question, but no visible recovery notice was rendered; this violates the workbook's required announced recovery behavior.</x:v>
+        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -5865,13 +5865,13 @@
         <x:v>Tab/focus and Enter/Space where applicable</x:v>
       </x:c>
       <x:c r="N21" s="72" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O21" s="70" t="str">
-        <x:v>Invalid/extra URL state normalized to the nearest valid question, but no visible recovery notice was rendered; this violates the workbook's required announced recovery behavior.</x:v>
+        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -5918,10 +5918,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O22" s="70" t="str">
-        <x:v>Objective bounds passed at 1440, 1024, 768, 390, and 320 widths; owner must judge visible focus ring, visual overlap, and settled scrolling.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the visible focus ring, visual overlap, and settled scrolling.</x:v>
       </x:c>
       <x:c r="P22" s="70" t="str">
-        <x:v>docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="84" customHeight="1">
@@ -5968,10 +5968,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O23" s="70" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P23" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -6018,10 +6018,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O24" s="71" t="str">
-        <x:v>Focused lifecycle suite and browser trace verified URL/state behavior for the covered transition; see row-specific recovery/keyboard findings.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P24" s="71" t="str">
-        <x:v>npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6050,7 +6050,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra560e367238a4829"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84bbf069371941a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6211,10 +6211,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -6261,10 +6261,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -6311,10 +6311,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -6361,10 +6361,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -6411,10 +6411,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -6461,10 +6461,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -6511,10 +6511,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -6561,10 +6561,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -6611,10 +6611,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -6661,10 +6661,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O14" s="70" t="str">
-        <x:v>Objective link/count/overflow/focus or static reduced-motion checks passed; owner must judge visual balance, focus-ring visibility, and settled motion behavior.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge mobile hub visual balance and focus-ring visibility.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -6711,10 +6711,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O15" s="70" t="str">
-        <x:v>Objective link/count/overflow/focus or static reduced-motion checks passed; owner must judge visual balance, focus-ring visibility, and settled motion behavior.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge focus-ring appearance and traversal feel.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -6761,10 +6761,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O16" s="70" t="str">
-        <x:v>Clipboard-available success feedback was verified; blocked-clipboard behavior was not forced. Owner must judge fallback feedback and lack of misleading persistence language.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge fallback feedback tone and lack of misleading persistence language.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -6811,10 +6811,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O17" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -6861,10 +6861,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O18" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -6911,10 +6911,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O19" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -6961,10 +6961,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O20" s="70" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -7011,10 +7011,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O21" s="70" t="str">
-        <x:v>Objective link/count/overflow/focus or static reduced-motion checks passed; owner must judge visual balance, focus-ring visibility, and settled motion behavior.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge reduced-motion settling and readability.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -7061,10 +7061,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O22" s="71" t="str">
-        <x:v>Review/regression suites and browser checks verified route/link/metadata behavior; visual portions remain owner-gated where marked.</x:v>
+        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P22" s="71" t="str">
-        <x:v>npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7093,7 +7093,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R801ea49300a8499d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b5da749c0a3449c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7254,10 +7254,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Prior evidence preserved; this execution phase does not treat subjective visual acceptance as automated Pass.</x:v>
+        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -7304,10 +7304,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Prior multi-select/copy evidence remains useful; current browser verified exact copy success, while fallback and generated-copy editorial issues remain open.</x:v>
+        <x:v>Retest passed exact visible-to-clipboard matching and truthful blocked feedback; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -7354,10 +7354,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Objective rules-safety or preserved-surface regression evidence was rechecked by evaluator/regression suites.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -7404,10 +7404,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Prior 320px overlap remediation remains recorded; current bounds pass, while owner visual acceptance remains open.</x:v>
+        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -7454,10 +7454,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Prior 390px readability evidence remains recorded; owner visual acceptance remains open.</x:v>
+        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -7504,10 +7504,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="71" t="str">
-        <x:v>Objective rules-safety or preserved-surface regression evidence was rechecked by evaluator/regression suites.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P10" s="71" t="str">
-        <x:v>docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -7554,10 +7554,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" t="str">
-        <x:v>Candidate authority matched before QA; workbook was restored from HEAD before execution.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P11" t="str">
-        <x:v>git status/rev-parse; workbook artifact-tool inspect</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: git status/rev-parse; workbook artifact-tool inspect</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -7601,13 +7601,13 @@
         <x:v>Browser automation plus keyboard attempt</x:v>
       </x:c>
       <x:c r="N12" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" t="str">
-        <x:v>The command suites passed where they ran, but independent evaluator/browser audits found repeated response fallback, semicolon-chain copy, and missing recovery notice.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P12" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; command outputs</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; command outputs</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -7654,10 +7654,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" t="str">
-        <x:v>Finding-a-Table deterministic evaluator coverage passed.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P13" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -7701,13 +7701,13 @@
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="N14" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O14" t="str">
-        <x:v>Generated-copy and option-ID defects recorded; no implementation was changed.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P14" t="str">
-        <x:v>docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -7751,13 +7751,13 @@
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="N15" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O15" t="str">
-        <x:v>Response-label fallback is a concrete defect; safety boundary itself passed.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P15" t="str">
-        <x:v>docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -7801,13 +7801,13 @@
         <x:v>Enter/Space attempt blocked</x:v>
       </x:c>
       <x:c r="N16" t="str">
-        <x:v>Automated Fail</x:v>
+        <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O16" t="str">
-        <x:v>Two recovery failures and one blocked keyboard-control path are recorded; no product changes made.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P16" t="str">
-        <x:v>docs/qa/evidence/finding-a-table-invalid-recovery.png; browser history/keyboard trace; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser history/keyboard trace; npm.cmd run test:strategium-lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -7854,10 +7854,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O17" t="str">
-        <x:v>Owner must judge visual balance, focus-ring appearance, reduced-motion settling, and mobile composition.</x:v>
+        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P17" t="str">
-        <x:v>docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; browser console trace</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; browser console trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -7904,10 +7904,410 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O18" t="str">
-        <x:v>Owner acceptance is not claimed; checklist is prepared for the remaining subjective gate.</x:v>
+        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P18" t="str">
-        <x:v>docs/qa/strategium-lifecycle-owner-acceptance-checklist.md</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>LOG-015</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>Retest identity</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Candidate implementation</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>Failed baseline implementation SHA and tested remediated implementation SHA</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>Baseline QA evidence commit 953a9052d2b056ed39051f11e247938fa60555d4 is preserved before product remediation.</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>Failed baseline 6f807816a81ca347cbd180a8c1ab413df84dce69; remediated implementation tested 84a458aa7b2c14db6184fc0b11271cbfeb7ed9b0; retest date 2026-07-31.</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Record the exact implementation commit under test and keep the later workbook commit separate.</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>Execution metadata</x:v>
+      </x:c>
+      <x:c r="J19" t="str">
+        <x:v>Retest ran against implementation commit 84a458aa7b2c14db6184fc0b11271cbfeb7ed9b0; this workbook does not replace that tested SHA with its later documentation commit.</x:v>
+      </x:c>
+      <x:c r="K19" t="str">
+        <x:v>Do not claim a later workbook commit was the implementation tested.</x:v>
+      </x:c>
+      <x:c r="L19" t="str">
+        <x:v>Desktop runtime</x:v>
+      </x:c>
+      <x:c r="M19" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="N19" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O19" t="str">
+        <x:v>Exact remediated implementation SHA recorded: 84a458aa7b2c14db6184fc0b11271cbfeb7ed9b0.</x:v>
+      </x:c>
+      <x:c r="P19" t="str">
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; QA baseline commit 953a9052d2b056ed39051f11e247938fa60555d4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>LOG-016</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>QA baseline preservation</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Candidate history</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>QA-baseline evidence commit</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>First-run evidence was intentionally dirty QA material and was committed before product edits.</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>QA baseline evidence commit 953a9052d2b056ed39051f11e247938fa60555d4; original candidate 6f807816a81ca347cbd180a8c1ab413df84dce69.</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>Preserve first-run evidence and record its commit before remediation.</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>Execution metadata</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>QA baseline evidence commit 953a9052d2b056ed39051f11e247938fa60555d4 preserves the failed run; no first-run evidence was overwritten or deleted.</x:v>
+      </x:c>
+      <x:c r="K20" t="str">
+        <x:v>No reset, discard, or evidence deletion.</x:v>
+      </x:c>
+      <x:c r="L20" t="str">
+        <x:v>Desktop runtime</x:v>
+      </x:c>
+      <x:c r="M20" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="N20" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O20" t="str">
+        <x:v>Baseline evidence commit is preserved and linked in the retest record.</x:v>
+      </x:c>
+      <x:c r="P20" t="str">
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>LOG-017</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>Retest command set</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>All lifecycle routes</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>Automated retest command set</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>Candidate implementation commit is fixed and candidate/control worktrees were clean before retest artifacts.</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>Focused lifecycle, review, lint, copy-boundaries, metadata, frontend-smoke, parser, browser-smoke, and full npm test suites.</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>Run the complete objective retest suite without editing implementation during validation.</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>Execution summary</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>All required objective command suites passed; full npm test exited 0.</x:v>
+      </x:c>
+      <x:c r="K21" t="str">
+        <x:v>No product implementation change during retest.</x:v>
+      </x:c>
+      <x:c r="L21" t="str">
+        <x:v>1440x900, 1024x768, 768x1024, 390x844, 320x568</x:v>
+      </x:c>
+      <x:c r="M21" t="str">
+        <x:v>Repository Puppeteer with Edge</x:v>
+      </x:c>
+      <x:c r="N21" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O21" t="str">
+        <x:v>Retest command set passed, including full repository test suite exit 0.</x:v>
+      </x:c>
+      <x:c r="P21" t="str">
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>LOG-018</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>Finding and Before evaluator audit</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>Finding a Table / Before the Game</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>Complete deterministic output coverage</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>Exact remediated implementation imported into the evaluator.</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>Finding 1,200 combinations; Before 1,935,360 reachable combinations including disclosure/agreement subsets.</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>Enumerate output categories, cards, grammar, punctuation, bracket omission, optional fields, disclosure retention, and copy-safe constraints.</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>Evaluator coverage</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>Finding: three categories, 100 explanations, five follow-ups, three mismatch warnings. Before: 1,935,360 combinations, max 434 characters, zero semicolon, malformed, lost-disclosure, unresolved-ID, or duplicate-clause outputs.</x:v>
+      </x:c>
+      <x:c r="K22" t="str">
+        <x:v>No score, certainty, player label, semicolon chain, placeholder, consent claim, or empty fragment.</x:v>
+      </x:c>
+      <x:c r="L22" t="str">
+        <x:v>Node evaluator</x:v>
+      </x:c>
+      <x:c r="M22" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="N22" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O22" t="str">
+        <x:v>Complete evaluator output space passed with no controlling Before-the-Game defects remaining.</x:v>
+      </x:c>
+      <x:c r="P22" t="str">
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>LOG-019</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>During response and safety audit</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>During the Game</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>All six moments and 48 response pairs</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>Canonical response catalog loaded from the remediated implementation.</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>6 entry moments x 8 response choices = 48 pairs.</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Verify selected response labels, response-specific guidance, four result concepts, official lookup/human adjudication routing, and safety boundaries.</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>Rules/safety audit</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>48 pairs exercised; zero fallback pairs and zero prohibited-content violations. Rules paths remain neutral and route toward official lookup or human adjudication.</x:v>
+      </x:c>
+      <x:c r="K23" t="str">
+        <x:v>No target, attack, removal, threat score, player rating, tactical sequencing, invented ruling, objective correctness, or manipulative table-politics advice.</x:v>
+      </x:c>
+      <x:c r="L23" t="str">
+        <x:v>Node evaluator + Puppeteer</x:v>
+      </x:c>
+      <x:c r="M23" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="N23" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O23" t="str">
+        <x:v>All 48 response mappings and the safety scan passed.</x:v>
+      </x:c>
+      <x:c r="P23" t="str">
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>LOG-020</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>Recovery, final action, and keyboard retest</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>All lifecycle routes</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>State recovery and native keyboard semantics</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>Direct Puppeteer/Edge runner replaced the first-run in-app keyboard limitation.</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>Partial, invalid, extra, and beyond-sequence state; final action; copy; Enter; Space; link Enter; ordinary history.</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>Verify visible polite recovery, no clean-route notice, named final result action, exact clipboard match, truthful fallback, native activation, focus visibility, and no trap.</x:v>
+      </x:c>
+      <x:c r="I24" t="str">
+        <x:v>State audit</x:v>
+      </x:c>
+      <x:c r="J24" t="str">
+        <x:v>All recovery classes announce and normalize safely; valid history stays quiet; final action builds the result directly; copy and native keyboard activation pass.</x:v>
+      </x:c>
+      <x:c r="K24" t="str">
+        <x:v>No modal trap, unsafe recovery, generic final Continue, or misleading copy feedback.</x:v>
+      </x:c>
+      <x:c r="L24" t="str">
+        <x:v>Repository Puppeteer + Edge</x:v>
+      </x:c>
+      <x:c r="M24" t="str">
+        <x:v>Enter, Space, Escape where relevant</x:v>
+      </x:c>
+      <x:c r="N24" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O24" t="str">
+        <x:v>QA-BLOCK-001 is resolved as a harness limitation: direct repository Puppeteer proves native Enter/Space/link activation and leaves no product keyboard defect.</x:v>
+      </x:c>
+      <x:c r="P24" t="str">
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; docs/qa/evidence/retest-01/before-final-action-390x844.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>LOG-021</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>Responsive and accessibility mechanics</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>All Strategium routes</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>Required viewports, names, focus, console, and network checks</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>Edge headless browser loaded the exact implementation.</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>1440x900, 1024x768, 768x1024, 390x844, 320x568; hub, initial routes, results, recovery, copy, Console and review regression suites.</x:v>
+      </x:c>
+      <x:c r="H25" t="str">
+        <x:v>Check overflow, clipping/overlap mechanics, focus bounds/styles, accessible control names, console errors, failed requests, and screenshots.</x:v>
+      </x:c>
+      <x:c r="I25" t="str">
+        <x:v>Responsive/accessibility</x:v>
+      </x:c>
+      <x:c r="J25" t="str">
+        <x:v>Zero horizontal-overflow or unnamed-control findings, zero console errors, zero failed requests, and screenshots captured at primary routes and mobile boundaries. Subjective visual comfort remains owner-gated.</x:v>
+      </x:c>
+      <x:c r="K25" t="str">
+        <x:v>No mechanically hidden control or console/network error.</x:v>
+      </x:c>
+      <x:c r="L25" t="str">
+        <x:v>All required viewports</x:v>
+      </x:c>
+      <x:c r="M25" t="str">
+        <x:v>Native semantics and focus styles</x:v>
+      </x:c>
+      <x:c r="N25" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O25" t="str">
+        <x:v>Objective responsive/accessibility mechanics passed; subjective visual composition remains in the existing 15-row owner set.</x:v>
+      </x:c>
+      <x:c r="P25" t="str">
+        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>LOG-022</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>Remaining owner-review scope</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>Strategium owner review</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>Subjective acceptance boundary and blocked condition</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>Objective retest completed with zero Automated Fail and zero Blocked rows.</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>15 existing Owner Review Required rows: hub balance, representative output tone, six During-the-Game moments, desktop/mobile sweep, After-the-Game, and Commander Console.</x:v>
+      </x:c>
+      <x:c r="H26" t="str">
+        <x:v>Hand the owner the focused checklist without asking for repeated technical matrix execution.</x:v>
+      </x:c>
+      <x:c r="I26" t="str">
+        <x:v>Owner acceptance subset</x:v>
+      </x:c>
+      <x:c r="J26" t="str">
+        <x:v>Only the remaining subjective visual/editorial/tone judgments remain; no blocked condition remains after direct keyboard validation.</x:v>
+      </x:c>
+      <x:c r="K26" t="str">
+        <x:v>Do not claim owner acceptance, independent review, certification, deployment, or integration.</x:v>
+      </x:c>
+      <x:c r="L26" t="str">
+        <x:v>Desktop/mobile</x:v>
+      </x:c>
+      <x:c r="M26" t="str">
+        <x:v>Owner physical review where listed</x:v>
+      </x:c>
+      <x:c r="N26" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O26" t="str">
+        <x:v>Remaining owner scope is limited to the 15 pre-existing subjective rows; Blocked count is zero.</x:v>
+      </x:c>
+      <x:c r="P26" t="str">
+        <x:v>docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; ${evidenceRoot}/retest-summary.json</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7920,17 +8320,20 @@
     <x:cfRule type="containsText" dxfId="16" priority="2" operator="containsText" text="Fail"/>
     <x:cfRule type="containsText" dxfId="17" priority="3" operator="containsText" text="Blocked"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="N5:N10">
       <x:formula1>"Not Run,Pass,Fail,Blocked,Not Applicable"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="N5:N11">
       <x:formula1>"Automated Pass,Automated Fail,Owner Review Required,Blocked"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="N5:N19">
+      <x:formula1>"Automated Pass,Automated Fail,Owner Review Required,Blocked"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24209cdef9fc47f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd8bbfc70eab40e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
qa(strategium): record final pregame copy retest
</commit_message>
<xml_diff>
--- a/docs/qa/Strategium_Game_Lifecycle_Human_QA_Workbook.xlsx
+++ b/docs/qa/Strategium_Game_Lifecycle_Human_QA_Workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfbc712df31b24a23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finding a Table" sheetId="2" r:id="Rfc9f3563732a4480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before the Game" sheetId="3" r:id="R68f89de66a404456"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="During the Game" sheetId="4" r:id="Re59c016ca24d4131"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="5" r:id="Racf911ef59ff422d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation and Regression" sheetId="6" r:id="Rf4bab47ab3b1484a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human QA Log" sheetId="7" r:id="R44321b2a17d04e72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra47dd2e177e54ed3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finding a Table" sheetId="2" r:id="R192f6bb63cf146d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before the Game" sheetId="3" r:id="Ra50d5aa4776e4a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="During the Game" sheetId="4" r:id="Rcbe7b1bbdad54e65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="5" r:id="Rbc55d29879e34267"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation and Regression" sheetId="6" r:id="Rbca985af9fc649ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human QA Log" sheetId="7" r:id="Rc43f0058c2374eb4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -968,8 +968,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="HumanQALog" displayName="HumanQALog" ref="A4:P26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:P26"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="HumanQALog" displayName="HumanQALog" ref="A4:P34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:P34"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Technique"/>
@@ -1246,7 +1246,7 @@
         <x:v>Exact remediated candidate SHA</x:v>
       </x:c>
       <x:c r="B5" s="52" t="str">
-        <x:v>84a458aa7b2c14db6184fc0b11271cbfeb7ed9b0</x:v>
+        <x:v>bc5dc696388bc7678e9efc9786c3b2d4985606b4</x:v>
       </x:c>
       <x:c r="C5" s="49"/>
       <x:c r="D5" s="53" t="str">
@@ -1354,7 +1354,7 @@
         <x:v>Candidate HEAD tested</x:v>
       </x:c>
       <x:c r="B11" s="83" t="str">
-        <x:v>84a458aa7b2c14db6184fc0b11271cbfeb7ed9b0</x:v>
+        <x:v>bc5dc696388bc7678e9efc9786c3b2d4985606b4</x:v>
       </x:c>
       <x:c r="C11" s="83"/>
       <x:c r="D11" s="54" t="str">
@@ -1362,7 +1362,7 @@
       </x:c>
       <x:c r="E11" s="84" t="n">
         <x:f>COUNTA('Human QA Log'!$A$5:$A$1000)</x:f>
-        <x:v>22</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F11" s="83"/>
       <x:c r="G11" s="83"/>
@@ -1563,7 +1563,7 @@
       </x:c>
       <x:c r="E20" s="87" t="n">
         <x:f>COUNTIF('Human QA Log'!$N$5:$N$1000,"Automated Pass")</x:f>
-        <x:v>16</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F20" s="87" t="n">
         <x:f>COUNTIF('Human QA Log'!$N$5:$N$1000,"Automated Fail")</x:f>
@@ -1792,7 +1792,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -1842,7 +1842,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -1892,7 +1892,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -1942,7 +1942,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -1992,7 +1992,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -2042,7 +2042,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -2092,7 +2092,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -2142,7 +2142,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -2192,7 +2192,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -2242,7 +2242,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -2292,7 +2292,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -2342,7 +2342,7 @@
         <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -2392,7 +2392,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -2442,7 +2442,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge readable composition, clipping, and visual comfort across the five supported viewports.</x:v>
       </x:c>
       <x:c r="P18" s="71" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2471,7 +2471,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98f7a90c19054fb6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a24a0a9e0394965"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2635,7 +2635,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -2685,7 +2685,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -2735,7 +2735,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -2785,7 +2785,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -2835,7 +2835,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -2885,7 +2885,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -2935,7 +2935,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -2985,7 +2985,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -3035,7 +3035,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -3085,7 +3085,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -3135,7 +3135,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -3185,7 +3185,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -3235,7 +3235,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -3285,7 +3285,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -3335,7 +3335,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -3385,7 +3385,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -3435,7 +3435,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -3485,7 +3485,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P22" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="84" customHeight="1">
@@ -3535,7 +3535,7 @@
         <x:v>Retest passed: None of these is mutually exclusive with every positive disclosure, and switching either direction clears the conflicting selections.</x:v>
       </x:c>
       <x:c r="P23" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -3585,7 +3585,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P24" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="84" customHeight="1">
@@ -3635,7 +3635,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P25" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="84" customHeight="1">
@@ -3685,7 +3685,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P26" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="84" customHeight="1">
@@ -3735,7 +3735,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P27" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="84" customHeight="1">
@@ -3785,7 +3785,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P28" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="84" customHeight="1">
@@ -3835,7 +3835,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P29" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="84" customHeight="1">
@@ -3885,7 +3885,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P30" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="84" customHeight="1">
@@ -3935,7 +3935,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the fallback-copy affordance and editorial naturalness after the exact success/blocked mechanics passed.</x:v>
       </x:c>
       <x:c r="P31" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="84" customHeight="1">
@@ -3985,7 +3985,7 @@
         <x:v>Retest passed: the final step uses the named primary Build my pregame statement action, remains disabled until valid, preserves Back and multi-select, and reaches the result directly.</x:v>
       </x:c>
       <x:c r="P32" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/before-game-final-step-continue.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/before-game-final-step-continue.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="84" customHeight="1">
@@ -4035,7 +4035,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge long-copy wrapping, result-card readability, and visual/editorial comfort.</x:v>
       </x:c>
       <x:c r="P33" s="71" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4064,7 +4064,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R675594daaa9b44a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1be7ddcbc864ca7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4228,7 +4228,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -4278,7 +4278,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -4328,7 +4328,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -4378,7 +4378,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -4428,7 +4428,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -4478,7 +4478,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -4528,7 +4528,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -4578,7 +4578,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -4628,7 +4628,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -4678,7 +4678,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -4728,7 +4728,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -4778,7 +4778,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -4828,7 +4828,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the thin-flow visual hierarchy and readability.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -4878,7 +4878,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P18" s="71" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4907,7 +4907,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re686c22b85d64246"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R521d531798c74eb1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5071,7 +5071,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -5121,7 +5121,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -5171,7 +5171,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -5221,7 +5221,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -5271,7 +5271,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -5321,7 +5321,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -5371,7 +5371,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -5421,7 +5421,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -5471,7 +5471,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -5521,7 +5521,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -5571,7 +5571,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -5621,7 +5621,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -5671,7 +5671,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -5721,7 +5721,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -5771,7 +5771,7 @@
         <x:v>Retest passed through direct repository Puppeteer: native buttons activated with Enter and Space, lifecycle link activated with Enter, focus remained visible, and the final action/copy action were keyboard-operable without a focus trap.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser keyboard trace; native button/link static inspection</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser keyboard trace; native button/link static inspection</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -5821,7 +5821,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -5871,7 +5871,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -5921,7 +5921,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the visible focus ring, visual overlap, and settled scrolling.</x:v>
       </x:c>
       <x:c r="P22" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="84" customHeight="1">
@@ -5971,7 +5971,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P23" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -6021,7 +6021,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P24" s="71" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6050,7 +6050,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84bbf069371941a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ac03fc2843c417b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6214,7 +6214,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -6264,7 +6264,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -6314,7 +6314,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -6364,7 +6364,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -6414,7 +6414,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -6464,7 +6464,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -6514,7 +6514,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -6564,7 +6564,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -6614,7 +6614,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -6664,7 +6664,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge mobile hub visual balance and focus-ring visibility.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -6714,7 +6714,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge focus-ring appearance and traversal feel.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -6764,7 +6764,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge fallback feedback tone and lack of misleading persistence language.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -6814,7 +6814,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -6864,7 +6864,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -6914,7 +6914,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -6964,7 +6964,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -7014,7 +7014,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge reduced-motion settling and readability.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -7064,7 +7064,7 @@
         <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P22" s="71" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7093,7 +7093,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b5da749c0a3449c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R988e06a80a9244d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7257,7 +7257,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -7307,7 +7307,7 @@
         <x:v>Retest passed exact visible-to-clipboard matching and truthful blocked feedback; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -7357,7 +7357,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -7407,7 +7407,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -7457,7 +7457,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -7507,7 +7507,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P10" s="71" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -7557,7 +7557,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P11" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: git status/rev-parse; workbook artifact-tool inspect</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: git status/rev-parse; workbook artifact-tool inspect</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -7607,7 +7607,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P12" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; command outputs</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; command outputs</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -7657,7 +7657,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P13" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -7707,7 +7707,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P14" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -7757,7 +7757,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P15" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -7807,7 +7807,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P16" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser history/keyboard trace; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser history/keyboard trace; npm.cmd run test:strategium-lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -7857,7 +7857,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P17" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; browser console trace</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; browser console trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -7907,7 +7907,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P18" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -7954,10 +7954,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O19" t="str">
-        <x:v>Exact remediated implementation SHA recorded: 84a458aa7b2c14db6184fc0b11271cbfeb7ed9b0.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P19" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; QA baseline commit 953a9052d2b056ed39051f11e247938fa60555d4</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; QA baseline commit 953a9052d2b056ed39051f11e247938fa60555d4</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -8004,10 +8004,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O20" t="str">
-        <x:v>Baseline evidence commit is preserved and linked in the retest record.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P20" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -8054,10 +8054,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O21" t="str">
-        <x:v>Retest command set passed, including full repository test suite exit 0.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P21" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -8104,10 +8104,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O22" t="str">
-        <x:v>Complete evaluator output space passed with no controlling Before-the-Game defects remaining.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P22" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -8154,10 +8154,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O23" t="str">
-        <x:v>All 48 response mappings and the safety scan passed.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P23" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -8204,10 +8204,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O24" t="str">
-        <x:v>QA-BLOCK-001 is resolved as a harness limitation: direct repository Puppeteer proves native Enter/Space/link activation and leaves no product keyboard defect.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P24" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; docs/qa/evidence/retest-01/before-final-action-390x844.png</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; docs/qa/evidence/retest-01/before-final-action-390x844.png</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -8254,10 +8254,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O25" t="str">
-        <x:v>Objective responsive/accessibility mechanics passed; subjective visual composition remains in the existing 15-row owner set.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P25" t="str">
-        <x:v>docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -8304,10 +8304,410 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O26" t="str">
-        <x:v>Remaining owner scope is limited to the 15 pre-existing subjective rows; Blocked count is zero.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P26" t="str">
-        <x:v>docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; ${evidenceRoot}/retest-summary.json</x:v>
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-01/retest-summary.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>LOG-023</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>Final copy retest identity</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>Before the Game</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>Previous final candidate and new implementation SHA</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>Previous final candidate 63b40ba0eac7a533f5401fa8018a183ba40b2d77; implementation retest target bc5dc696388bc7678e9efc9786c3b2d4985606b4; retest date 2026-07-31.</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>Implementation commit bc5dc696388bc7678e9efc9786c3b2d4985606b4 is the exact code under test; the later workbook commit remains documentation only.</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>Record the implementation SHA actually tested and preserve the prior final candidate.</x:v>
+      </x:c>
+      <x:c r="I27" t="str">
+        <x:v>Execution metadata</x:v>
+      </x:c>
+      <x:c r="J27" t="str">
+        <x:v>Retest executed against bc5dc696388bc7678e9efc9786c3b2d4985606b4 after previous final candidate 63b40ba0eac7a533f5401fa8018a183ba40b2d77.</x:v>
+      </x:c>
+      <x:c r="K27" t="str">
+        <x:v>Do not substitute a later QA/docs commit for the tested implementation SHA.</x:v>
+      </x:c>
+      <x:c r="L27" t="str">
+        <x:v>Desktop runtime</x:v>
+      </x:c>
+      <x:c r="M27" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="N27" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O27" t="str">
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+      </x:c>
+      <x:c r="P27" t="str">
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; Previous retest: docs/qa/evidence/retest-01/retest-summary.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>LOG-024</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>Expanded Before-the-Game copy audit</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>Before the Game</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>Complete reachable generated-copy space</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>Exact remediated implementation imported by the evaluator.</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>1,935,360 combinations across brackets, deck behavior, finish, timing, disclosure subsets, and final-agreement subsets.</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>Check grammar, capitalization, list punctuation, disclosure retention, sentence cap, semicolon absence, option-ID absence, and hard length boundary.</x:v>
+      </x:c>
+      <x:c r="I28" t="str">
+        <x:v>Evaluator coverage</x:v>
+      </x:c>
+      <x:c r="J28" t="str">
+        <x:v>All 1,935,360 statements passed; maximum 354 characters; preferred limit 300 with 92,923 large-disclosure boundary exceedances; hard limit 360; zero lowercase openings, incorrect conjunctions, repeated conjunctions, malformed list punctuation, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, malformed outputs, or statements above two sentences.</x:v>
+      </x:c>
+      <x:c r="K28" t="str">
+        <x:v>No broken phrase, empty optional fragment, repeated punctuation, semicolon chain, hidden high-impact disclosure, or overlong statement.</x:v>
+      </x:c>
+      <x:c r="L28" t="str">
+        <x:v>Bundled Node evaluator</x:v>
+      </x:c>
+      <x:c r="M28" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="N28" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O28" t="str">
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+      </x:c>
+      <x:c r="P28" t="str">
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>LOG-025</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>Disclosure retention and list composition</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>Before the Game</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>Every disclosure remains lossless and readable</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>Canonical disclosure catalog and shared natural-list formatter are loaded.</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>All positive disclosure subsets, None-of-these transitions, every agreement combination, and 12 risk-based representative samples.</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>Verify explicit high-impact wording, correct extra-turn/long-turn conjunction, human-readable list joining, and result-card losslessness.</x:v>
+      </x:c>
+      <x:c r="I29" t="str">
+        <x:v>Copy composition</x:v>
+      </x:c>
+      <x:c r="J29" t="str">
+        <x:v>Zero lost disclosures, zero incorrect 'or' joins, zero repeated-conjunction lists, zero malformed list punctuation; compact samples cover no disclosures plus each agreement, fast mana/tutors/combo, extra turns/long turns, all high-impact categories, proxies dual-use, unsure bracket, not using brackets, and still figuring it out.</x:v>
+      </x:c>
+      <x:c r="K29" t="str">
+        <x:v>No selected category disappears or is hidden by grouping.</x:v>
+      </x:c>
+      <x:c r="L29" t="str">
+        <x:v>Bundled Node evaluator</x:v>
+      </x:c>
+      <x:c r="M29" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="N29" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O29" t="str">
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+      </x:c>
+      <x:c r="P29" t="str">
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>LOG-026</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>During response and lifecycle regression</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>During the Game / lifecycle</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>All six moments, 48 response pairs, and route regressions</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>Canonical response catalog and exact implementation loaded.</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>Six entry moments x eight responses; Finding 1,200 combinations; route/recovery/history checks; After-the-Game and Console regression suites.</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>Verify selected response guidance, safety boundaries, route behavior, and unchanged adjacent surfaces.</x:v>
+      </x:c>
+      <x:c r="I30" t="str">
+        <x:v>Regression coverage</x:v>
+      </x:c>
+      <x:c r="J30" t="str">
+        <x:v>All 48 During-the-Game pairs passed with zero fallback and zero safety violations; Finding remains 1,200 combinations with varied categories/copy; review suite and route regressions passed.</x:v>
+      </x:c>
+      <x:c r="K30" t="str">
+        <x:v>No target, threat score, player rating, tactical advice, invented ruling, objective-correctness claim, or stale route label.</x:v>
+      </x:c>
+      <x:c r="L30" t="str">
+        <x:v>Bundled Node + repository tests</x:v>
+      </x:c>
+      <x:c r="M30" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="N30" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O30" t="str">
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+      </x:c>
+      <x:c r="P30" t="str">
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-review; npm.cmd run test:strategium-lifecycle</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>LOG-027</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>Clipboard and final action</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>Before the Game</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>Exact copy action and direct result navigation</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>Generated result and native controls are reachable in the Edge runner.</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>Named final action, Back, multi-select, visible statement, clipboard success, and blocked clipboard paths.</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>Verify exact visible-to-clipboard match, truthful success/blocked feedback, no generic final Continue, and direct result build.</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>Interaction mechanics</x:v>
+      </x:c>
+      <x:c r="J31" t="str">
+        <x:v>Exact visible statement copied; success says 'Copied for the table.'; blocked clipboard says 'Select the sentence above to copy it.'; final action is primary, named, and reaches result directly.</x:v>
+      </x:c>
+      <x:c r="K31" t="str">
+        <x:v>No mismatched clipboard text, misleading feedback, redundant Continue, or focus trap.</x:v>
+      </x:c>
+      <x:c r="L31" t="str">
+        <x:v>Microsoft Edge via Puppeteer</x:v>
+      </x:c>
+      <x:c r="M31" t="str">
+        <x:v>Enter and Space</x:v>
+      </x:c>
+      <x:c r="N31" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O31" t="str">
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+      </x:c>
+      <x:c r="P31" t="str">
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-final-action-390x844.png; docs/qa/evidence/retest-02/before-game-result-320x568.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>LOG-028</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>Responsive and accessibility mechanics</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>All Strategium routes</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>Required viewport, focus, console, and network checks</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>Edge headless browser loaded the exact implementation.</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>1440x900, 1024x768, 768x1024, 390x844, 320x568; hub, results, recovery, copy, Console and review paths.</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>Check overflow, accessible names, visible focus, native activation, heading transitions, console errors, failed requests, and screenshots.</x:v>
+      </x:c>
+      <x:c r="I32" t="str">
+        <x:v>Responsive/accessibility</x:v>
+      </x:c>
+      <x:c r="J32" t="str">
+        <x:v>Zero horizontal overflow, unnamed controls, console errors, and failed requests; screenshots captured for hub, primary routes, result, mobile, and recovery. Subjective visual comfort remains owner-gated.</x:v>
+      </x:c>
+      <x:c r="K32" t="str">
+        <x:v>No mechanically hidden control, network failure, or keyboard trap.</x:v>
+      </x:c>
+      <x:c r="L32" t="str">
+        <x:v>All required viewports</x:v>
+      </x:c>
+      <x:c r="M32" t="str">
+        <x:v>Native semantics; Enter and Space</x:v>
+      </x:c>
+      <x:c r="N32" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O32" t="str">
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+      </x:c>
+      <x:c r="P32" t="str">
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>LOG-029</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>Full repository validation</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>Repository regression</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>Focused, mandated, lint, and browser command set</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>Candidate was clean before QA artifact generation; product implementation was not changed during validation.</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>Lifecycle, review, copy-boundaries, route-metadata, frontend-smoke, parser, browser-smoke, lint, and full npm test.</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>Run all objective suites and retain exact results.</x:v>
+      </x:c>
+      <x:c r="I33" t="str">
+        <x:v>Execution summary</x:v>
+      </x:c>
+      <x:c r="J33" t="str">
+        <x:v>All command suites passed; npm.cmd test exited 0; no product source was changed during the retest.</x:v>
+      </x:c>
+      <x:c r="K33" t="str">
+        <x:v>No implementation remediation during validation.</x:v>
+      </x:c>
+      <x:c r="L33" t="str">
+        <x:v>Desktop runtime</x:v>
+      </x:c>
+      <x:c r="M33" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="N33" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O33" t="str">
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+      </x:c>
+      <x:c r="P33" t="str">
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:copy-boundaries; npm.cmd run test:route-metadata; npm.cmd run test:frontend-smoke; npm.cmd run test:parser; npm.cmd run test:browser-smoke; npm.cmd test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>LOG-030</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>Remaining owner gate</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>Strategium owner acceptance</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>Subjective acceptance boundary and blocked condition</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>Objective retest completed with zero Automated Fail and zero Blocked rows.</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>15 existing Owner Review Required cases covering hub balance, representative outputs, six During moments, desktop/mobile, After-the-Game, and Commander Console.</x:v>
+      </x:c>
+      <x:c r="H34" t="str">
+        <x:v>Hand off only the focused owner checklist; do not ask for repeated technical matrix execution.</x:v>
+      </x:c>
+      <x:c r="I34" t="str">
+        <x:v>Owner acceptance subset</x:v>
+      </x:c>
+      <x:c r="J34" t="str">
+        <x:v>Fifteen Owner Review Required cases remain for visual, editorial, tone, and physical-environment judgment; no blocked condition remains.</x:v>
+      </x:c>
+      <x:c r="K34" t="str">
+        <x:v>Do not claim owner acceptance, independent review, certification, deployment, integration, or push.</x:v>
+      </x:c>
+      <x:c r="L34" t="str">
+        <x:v>Desktop/mobile</x:v>
+      </x:c>
+      <x:c r="M34" t="str">
+        <x:v>Owner review where listed</x:v>
+      </x:c>
+      <x:c r="N34" t="str">
+        <x:v>Automated Pass</x:v>
+      </x:c>
+      <x:c r="O34" t="str">
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+      </x:c>
+      <x:c r="P34" t="str">
+        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-02/retest-summary.json</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8320,7 +8720,7 @@
     <x:cfRule type="containsText" dxfId="16" priority="2" operator="containsText" text="Fail"/>
     <x:cfRule type="containsText" dxfId="17" priority="3" operator="containsText" text="Blocked"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="3">
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="N5:N10">
       <x:formula1>"Not Run,Pass,Fail,Blocked,Not Applicable"</x:formula1>
     </x:dataValidation>
@@ -8330,10 +8730,16 @@
     <x:dataValidation type="list" sqref="N5:N19">
       <x:formula1>"Automated Pass,Automated Fail,Owner Review Required,Blocked"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="N5:N27">
+      <x:formula1>"Automated Pass,Automated Fail,Owner Review Required,Blocked"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="N5:N35">
+      <x:formula1>"Automated Pass,Automated Fail,Owner Review Required,Blocked"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd8bbfc70eab40e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25fe6da2107449ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
qa(strategium): record final owner remediation evidence
</commit_message>
<xml_diff>
--- a/docs/qa/Strategium_Game_Lifecycle_Human_QA_Workbook.xlsx
+++ b/docs/qa/Strategium_Game_Lifecycle_Human_QA_Workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra47dd2e177e54ed3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finding a Table" sheetId="2" r:id="R192f6bb63cf146d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before the Game" sheetId="3" r:id="Ra50d5aa4776e4a8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="During the Game" sheetId="4" r:id="Rcbe7b1bbdad54e65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="5" r:id="Rbc55d29879e34267"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation and Regression" sheetId="6" r:id="Rbca985af9fc649ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human QA Log" sheetId="7" r:id="Rc43f0058c2374eb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra52342a716164fe7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finding a Table" sheetId="2" r:id="Raef631e7c4e94531"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before the Game" sheetId="3" r:id="R453924abe6e243f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="During the Game" sheetId="4" r:id="R3ea7273c2bb746f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="5" r:id="R5d0e91217f45421d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation and Regression" sheetId="6" r:id="Rf312bc4823d2466a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human QA Log" sheetId="7" r:id="R9b56f95dd80745a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -968,8 +968,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="HumanQALog" displayName="HumanQALog" ref="A4:P34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:P34"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="HumanQALog" displayName="HumanQALog" ref="A4:P39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:P39"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Technique"/>
@@ -1246,7 +1246,7 @@
         <x:v>Exact remediated candidate SHA</x:v>
       </x:c>
       <x:c r="B5" s="52" t="str">
-        <x:v>bc5dc696388bc7678e9efc9786c3b2d4985606b4</x:v>
+        <x:v>03569c28644e40c39cd836b8e2559a652914d006</x:v>
       </x:c>
       <x:c r="C5" s="49"/>
       <x:c r="D5" s="53" t="str">
@@ -1335,7 +1335,7 @@
         <x:v>Execution status after automated retest</x:v>
       </x:c>
       <x:c r="B10" s="55" t="str">
-        <x:v>Objective rows are updated with the latest retest status. Automated Fail: 0. Blocked: 0. Fifteen subjective rows remain Owner Review Required; owner acceptance is not claimed.</x:v>
+        <x:v>Objective rows are updated with the latest owner-remediation retest. Automated Fail: 0. Blocked: 0. Twenty populated records remain Owner Review Required (15 prior subjective rows plus five OAR dispositions); owner acceptance is not claimed.</x:v>
       </x:c>
       <x:c r="C10" s="83"/>
       <x:c r="D10" s="54" t="str">
@@ -1354,7 +1354,7 @@
         <x:v>Candidate HEAD tested</x:v>
       </x:c>
       <x:c r="B11" s="83" t="str">
-        <x:v>bc5dc696388bc7678e9efc9786c3b2d4985606b4</x:v>
+        <x:v>03569c28644e40c39cd836b8e2559a652914d006</x:v>
       </x:c>
       <x:c r="C11" s="83"/>
       <x:c r="D11" s="54" t="str">
@@ -1362,7 +1362,7 @@
       </x:c>
       <x:c r="E11" s="84" t="n">
         <x:f>COUNTA('Human QA Log'!$A$5:$A$1000)</x:f>
-        <x:v>30</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F11" s="83"/>
       <x:c r="G11" s="83"/>
@@ -1571,7 +1571,7 @@
       </x:c>
       <x:c r="G20" s="87" t="n">
         <x:f>COUNTIF('Human QA Log'!$N$5:$N$1000,"Owner Review Required")</x:f>
-        <x:v>6</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H20" s="82" t="n">
         <x:f>COUNTIF('Human QA Log'!$N$5:$N$1000,"Blocked")</x:f>
@@ -1789,10 +1789,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -1839,10 +1839,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -1889,10 +1889,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -1939,10 +1939,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -1989,10 +1989,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -2039,10 +2039,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -2089,10 +2089,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -2139,10 +2139,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -2189,10 +2189,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -2239,10 +2239,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O14" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -2289,10 +2289,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O15" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -2339,10 +2339,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O16" s="70" t="str">
-        <x:v>Retest passed: 1,200 combinations produced all three categories, five cards, 100 explanations, five follow-up variants, and three mismatch warnings without score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -2392,7 +2392,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -2442,7 +2442,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge readable composition, clipping, and visual comfort across the five supported viewports.</x:v>
       </x:c>
       <x:c r="P18" s="71" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2471,7 +2471,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a24a0a9e0394965"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0d23498b8ac4b4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2635,7 +2635,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -2685,7 +2685,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -2735,7 +2735,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -2785,7 +2785,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -2835,7 +2835,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -2885,7 +2885,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -2935,7 +2935,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -2985,7 +2985,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -3035,7 +3035,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -3085,7 +3085,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -3135,7 +3135,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -3185,7 +3185,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -3235,7 +3235,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -3285,7 +3285,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -3335,7 +3335,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -3385,7 +3385,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -3435,7 +3435,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -3485,7 +3485,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P22" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="84" customHeight="1">
@@ -3535,7 +3535,7 @@
         <x:v>Retest passed: None of these is mutually exclusive with every positive disclosure, and switching either direction clears the conflicting selections.</x:v>
       </x:c>
       <x:c r="P23" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -3585,7 +3585,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P24" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="84" customHeight="1">
@@ -3635,7 +3635,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P25" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="84" customHeight="1">
@@ -3685,7 +3685,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P26" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="84" customHeight="1">
@@ -3735,7 +3735,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P27" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="84" customHeight="1">
@@ -3785,7 +3785,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P28" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="84" customHeight="1">
@@ -3835,7 +3835,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P29" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="84" customHeight="1">
@@ -3885,7 +3885,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
       </x:c>
       <x:c r="P30" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="84" customHeight="1">
@@ -3935,7 +3935,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the fallback-copy affordance and editorial naturalness after the exact success/blocked mechanics passed.</x:v>
       </x:c>
       <x:c r="P31" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; docs/qa/evidence/owner-remediation-01/console-log.txt; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="84" customHeight="1">
@@ -3985,7 +3985,7 @@
         <x:v>Retest passed: the final step uses the named primary Build my pregame statement action, remains disabled until valid, preserves Back and multi-select, and reaches the result directly.</x:v>
       </x:c>
       <x:c r="P32" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/before-game-final-step-continue.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/before-game-final-step-continue.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="84" customHeight="1">
@@ -4035,7 +4035,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge long-copy wrapping, result-card readability, and visual/editorial comfort.</x:v>
       </x:c>
       <x:c r="P33" s="71" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4064,7 +4064,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1be7ddcbc864ca7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R304adcc5348c4684"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4228,7 +4228,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -4278,7 +4278,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -4328,7 +4328,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -4378,7 +4378,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -4428,7 +4428,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -4478,7 +4478,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -4528,7 +4528,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -4578,7 +4578,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -4628,7 +4628,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -4678,7 +4678,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -4728,7 +4728,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -4778,7 +4778,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -4828,7 +4828,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the thin-flow visual hierarchy and readability.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -4878,7 +4878,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P18" s="71" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4907,7 +4907,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R521d531798c74eb1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf4d0028ec9b4993"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5071,7 +5071,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -5121,7 +5121,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -5171,7 +5171,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -5221,7 +5221,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -5271,7 +5271,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -5321,7 +5321,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -5371,7 +5371,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -5421,7 +5421,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -5471,7 +5471,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -5521,7 +5521,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -5571,7 +5571,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -5621,7 +5621,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -5671,7 +5671,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -5721,7 +5721,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -5771,7 +5771,7 @@
         <x:v>Retest passed through direct repository Puppeteer: native buttons activated with Enter and Space, lifecycle link activated with Enter, focus remained visible, and the final action/copy action were keyboard-operable without a focus trap.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser keyboard trace; native button/link static inspection</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser keyboard trace; native button/link static inspection</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -5821,7 +5821,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -5871,7 +5871,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -5921,7 +5921,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the visible focus ring, visual overlap, and settled scrolling.</x:v>
       </x:c>
       <x:c r="P22" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="84" customHeight="1">
@@ -5971,7 +5971,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P23" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -6021,7 +6021,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
       </x:c>
       <x:c r="P24" s="71" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6050,7 +6050,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ac03fc2843c417b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7214eb9fef844848"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6211,10 +6211,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -6261,10 +6261,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -6311,10 +6311,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -6361,10 +6361,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -6411,10 +6411,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -6461,10 +6461,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -6511,10 +6511,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -6561,10 +6561,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -6611,10 +6611,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -6664,7 +6664,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge mobile hub visual balance and focus-ring visibility.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -6714,7 +6714,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge focus-ring appearance and traversal feel.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -6764,7 +6764,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge fallback feedback tone and lack of misleading persistence language.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; docs/qa/evidence/owner-remediation-01/console-log.txt; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -6811,10 +6811,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O17" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -6861,10 +6861,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O18" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -6911,10 +6911,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O19" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -6961,10 +6961,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O20" s="70" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -7014,7 +7014,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge reduced-motion settling and readability.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -7061,10 +7061,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O22" s="71" t="str">
-        <x:v>Retest passed: lifecycle hub links, direct After-the-Game entry, Commander Console, global navigation, canonical metadata, no stale In development labels, no dead ends, mobile overflow, and preserved After-the-Game behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
       </x:c>
       <x:c r="P22" s="71" t="str">
-        <x:v>docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7093,7 +7093,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R988e06a80a9244d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a82cce515c741b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7257,7 +7257,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -7307,7 +7307,7 @@
         <x:v>Retest passed exact visible-to-clipboard matching and truthful blocked feedback; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -7357,7 +7357,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -7407,7 +7407,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -7457,7 +7457,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -7507,7 +7507,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P10" s="71" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -7557,7 +7557,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P11" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: git status/rev-parse; workbook artifact-tool inspect</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: git status/rev-parse; workbook artifact-tool inspect</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -7607,7 +7607,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P12" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; command outputs</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; command outputs</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -7657,7 +7657,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P13" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -7707,7 +7707,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P14" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -7757,7 +7757,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P15" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -7807,7 +7807,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
       </x:c>
       <x:c r="P16" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser history/keyboard trace; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser history/keyboard trace; npm.cmd run test:strategium-lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -7857,7 +7857,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P17" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; browser console trace</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; browser console trace</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -7907,7 +7907,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
       </x:c>
       <x:c r="P18" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -7957,7 +7957,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P19" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; QA baseline commit 953a9052d2b056ed39051f11e247938fa60555d4</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; QA baseline commit 953a9052d2b056ed39051f11e247938fa60555d4</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -8007,7 +8007,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P20" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -8057,7 +8057,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P21" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -8107,7 +8107,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P22" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -8157,7 +8157,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P23" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -8207,7 +8207,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P24" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; docs/qa/evidence/retest-01/before-final-action-390x844.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; docs/qa/evidence/retest-01/before-final-action-390x844.png</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -8257,7 +8257,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P25" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -8307,7 +8307,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P26" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-01/retest-summary.json</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-01/retest-summary.json</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -8357,7 +8357,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P27" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; Previous retest: docs/qa/evidence/retest-01/retest-summary.json</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; Previous retest: docs/qa/evidence/retest-01/retest-summary.json</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -8407,7 +8407,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P28" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -8457,7 +8457,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P29" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -8507,7 +8507,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P30" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-review; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-review; npm.cmd run test:strategium-lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -8557,7 +8557,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P31" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-final-action-390x844.png; docs/qa/evidence/retest-02/before-game-result-320x568.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-final-action-390x844.png; docs/qa/evidence/retest-02/before-game-result-320x568.png</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -8607,7 +8607,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P32" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -8657,7 +8657,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P33" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:copy-boundaries; npm.cmd run test:route-metadata; npm.cmd run test:frontend-smoke; npm.cmd run test:parser; npm.cmd run test:browser-smoke; npm.cmd test</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:copy-boundaries; npm.cmd run test:route-metadata; npm.cmd run test:frontend-smoke; npm.cmd run test:parser; npm.cmd run test:browser-smoke; npm.cmd test</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -8707,7 +8707,257 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
       </x:c>
       <x:c r="P34" t="str">
-        <x:v>Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-02/retest-summary.json</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-02/retest-summary.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>OAR-01</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>Commander Console hub preview balance</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>Navigation and Regression</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>OAR-01 visible owner defect</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>Rejected candidate affbd46be443d18d73a7a8a9bb9938dee36f5a34 lacked the compact 2x2 Console preview grid.</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>Four non-interactive previews are rendered: Pod Readiness, Archetypes, Threat &amp; Pressure, and Color Expectations. Browser assertions and desktop/mobile screenshots passed.</x:v>
+      </x:c>
+      <x:c r="H35" t="str">
+        <x:v>Owner judges balance, density, and whether previews read as useful non-routes.</x:v>
+      </x:c>
+      <x:c r="I35" t="str">
+        <x:v>Owner remediation disposition</x:v>
+      </x:c>
+      <x:c r="J35" t="str">
+        <x:v>Objective rendered presence and responsive mechanics passed; visual acceptance remains owner-gated.</x:v>
+      </x:c>
+      <x:c r="K35" t="str">
+        <x:v>Do not mark owner acceptance as passed.</x:v>
+      </x:c>
+      <x:c r="L35" t="str">
+        <x:v>1440x900 and 390x844</x:v>
+      </x:c>
+      <x:c r="M35" t="str">
+        <x:v>Not applicable to non-interactive previews</x:v>
+      </x:c>
+      <x:c r="N35" t="str">
+        <x:v>Owner Review Required</x:v>
+      </x:c>
+      <x:c r="O35" t="str">
+        <x:v>OAR-01 remediated; owner re-review required.</x:v>
+      </x:c>
+      <x:c r="P35" t="str">
+        <x:v>docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>OAR-02</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>Finding a Table result duplication</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>Finding a Table</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>OAR-02 visible owner defect</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>Rejected candidate affbd46be443d18d73a7a8a9bb9938dee36f5a34 repeated the compatibility conclusion in the hero and Provisional compatibility read card.</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>The duplicate card is removed; all 1,200 combinations remain valid; four required cards and interpreted explanation copy are asserted in the rendered result.</x:v>
+      </x:c>
+      <x:c r="H36" t="str">
+        <x:v>Owner judges whether the result hierarchy and interpretation read naturally.</x:v>
+      </x:c>
+      <x:c r="I36" t="str">
+        <x:v>Owner remediation disposition</x:v>
+      </x:c>
+      <x:c r="J36" t="str">
+        <x:v>Objective rendered structure and deterministic evaluator coverage passed; editorial acceptance remains owner-gated.</x:v>
+      </x:c>
+      <x:c r="K36" t="str">
+        <x:v>Do not mark owner acceptance as passed.</x:v>
+      </x:c>
+      <x:c r="L36" t="str">
+        <x:v>1440x900</x:v>
+      </x:c>
+      <x:c r="M36" t="str">
+        <x:v>Native result navigation</x:v>
+      </x:c>
+      <x:c r="N36" t="str">
+        <x:v>Owner Review Required</x:v>
+      </x:c>
+      <x:c r="O36" t="str">
+        <x:v>OAR-02 remediated; owner re-review required.</x:v>
+      </x:c>
+      <x:c r="P36" t="str">
+        <x:v>docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>OAR-03</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>Before-the-Game bracket selector</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>Before the Game</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>OAR-03 visible owner defect</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>Rejected candidate affbd46be443d18d73a7a8a9bb9938dee36f5a34 rendered seven visually heavy bracket cards with repeated notes.</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>Five compact accessible number controls plus distinct unsure/not-using choices are rendered; all seven states, selection, native semantics, and responsive behavior passed.</x:v>
+      </x:c>
+      <x:c r="H37" t="str">
+        <x:v>Owner judges visual clarity and whether the compact selector communicates without teaching definitions.</x:v>
+      </x:c>
+      <x:c r="I37" t="str">
+        <x:v>Owner remediation disposition</x:v>
+      </x:c>
+      <x:c r="J37" t="str">
+        <x:v>Objective rendered controls and mechanics passed; visual acceptance remains owner-gated.</x:v>
+      </x:c>
+      <x:c r="K37" t="str">
+        <x:v>Do not mark owner acceptance as passed.</x:v>
+      </x:c>
+      <x:c r="L37" t="str">
+        <x:v>1440x900 and 390x844</x:v>
+      </x:c>
+      <x:c r="M37" t="str">
+        <x:v>Enter and Space</x:v>
+      </x:c>
+      <x:c r="N37" t="str">
+        <x:v>Owner Review Required</x:v>
+      </x:c>
+      <x:c r="O37" t="str">
+        <x:v>OAR-03 remediated; owner re-review required.</x:v>
+      </x:c>
+      <x:c r="P37" t="str">
+        <x:v>docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>OAR-04</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>Before-the-Game action hierarchy</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>Before the Game</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>OAR-04 visible owner defect</x:v>
+      </x:c>
+      <x:c r="F38" t="str">
+        <x:v>Rejected candidate affbd46be443d18d73a7a8a9bb9938dee36f5a34 showed an unclear Step 5 Continue and detached Step 6 action bar.</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
+        <x:v>Step 5 uses Continue to final check in the standard footer; Step 6 has one gold Build my pregame statement footer action with Back and Start over; gating and direct result behavior passed.</x:v>
+      </x:c>
+      <x:c r="H38" t="str">
+        <x:v>Owner judges hierarchy, readability, and visual comfort of the unified footer.</x:v>
+      </x:c>
+      <x:c r="I38" t="str">
+        <x:v>Owner remediation disposition</x:v>
+      </x:c>
+      <x:c r="J38" t="str">
+        <x:v>Objective DOM placement, labels, native activation, selection gating, and mobile overflow passed; visual acceptance remains owner-gated.</x:v>
+      </x:c>
+      <x:c r="K38" t="str">
+        <x:v>Do not mark owner acceptance as passed.</x:v>
+      </x:c>
+      <x:c r="L38" t="str">
+        <x:v>1440x900 and 390x844</x:v>
+      </x:c>
+      <x:c r="M38" t="str">
+        <x:v>Enter and Space</x:v>
+      </x:c>
+      <x:c r="N38" t="str">
+        <x:v>Owner Review Required</x:v>
+      </x:c>
+      <x:c r="O38" t="str">
+        <x:v>OAR-04 remediated; owner re-review required.</x:v>
+      </x:c>
+      <x:c r="P38" t="str">
+        <x:v>docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>OAR-05</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>After-the-Game direct entry</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>Navigation and Regression</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>OAR-05 visible owner defect</x:v>
+      </x:c>
+      <x:c r="F39" t="str">
+        <x:v>Rejected candidate affbd46be443d18d73a7a8a9bb9938dee36f5a34 still opened the obsolete lifecycle selector from the hub.</x:v>
+      </x:c>
+      <x:c r="G39" t="str">
+        <x:v>The hub click path opens What best describes the game? directly; legacy selector URLs normalize safely; stale selector text is absent; existing review results remain green.</x:v>
+      </x:c>
+      <x:c r="H39" t="str">
+        <x:v>Owner judges continuity with the completed review experience and visual entry transition.</x:v>
+      </x:c>
+      <x:c r="I39" t="str">
+        <x:v>Owner remediation disposition</x:v>
+      </x:c>
+      <x:c r="J39" t="str">
+        <x:v>Objective hub-click route assertions, stale-copy absence, legacy recovery, history, focus, and result behavior passed; visual acceptance remains owner-gated.</x:v>
+      </x:c>
+      <x:c r="K39" t="str">
+        <x:v>Do not mark owner acceptance as passed.</x:v>
+      </x:c>
+      <x:c r="L39" t="str">
+        <x:v>1440x900</x:v>
+      </x:c>
+      <x:c r="M39" t="str">
+        <x:v>Native link activation</x:v>
+      </x:c>
+      <x:c r="N39" t="str">
+        <x:v>Owner Review Required</x:v>
+      </x:c>
+      <x:c r="O39" t="str">
+        <x:v>OAR-05 remediated; owner re-review required.</x:v>
+      </x:c>
+      <x:c r="P39" t="str">
+        <x:v>docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8739,7 +8989,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25fe6da2107449ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90f05ba0cfaf41ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
qa(strategium): record final runtime owner UX retest
</commit_message>
<xml_diff>
--- a/docs/qa/Strategium_Game_Lifecycle_Human_QA_Workbook.xlsx
+++ b/docs/qa/Strategium_Game_Lifecycle_Human_QA_Workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra52342a716164fe7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finding a Table" sheetId="2" r:id="Raef631e7c4e94531"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before the Game" sheetId="3" r:id="R453924abe6e243f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="During the Game" sheetId="4" r:id="R3ea7273c2bb746f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="5" r:id="R5d0e91217f45421d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation and Regression" sheetId="6" r:id="Rf312bc4823d2466a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human QA Log" sheetId="7" r:id="R9b56f95dd80745a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6ee11ef2981b4a5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finding a Table" sheetId="2" r:id="Re84f4b4f0d884a0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before the Game" sheetId="3" r:id="Rf46205a643a34ddc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="During the Game" sheetId="4" r:id="R6e1dc0e283a5497e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="5" r:id="R17d67ef50b684a42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation and Regression" sheetId="6" r:id="Rbff4c7a5113c4936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human QA Log" sheetId="7" r:id="R9f5c3af32f614418"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1246,7 +1246,7 @@
         <x:v>Exact remediated candidate SHA</x:v>
       </x:c>
       <x:c r="B5" s="52" t="str">
-        <x:v>03569c28644e40c39cd836b8e2559a652914d006</x:v>
+        <x:v>b9814549911306cc46ce6db321e0e2f4c354c4ec</x:v>
       </x:c>
       <x:c r="C5" s="49"/>
       <x:c r="D5" s="53" t="str">
@@ -1335,7 +1335,7 @@
         <x:v>Execution status after automated retest</x:v>
       </x:c>
       <x:c r="B10" s="55" t="str">
-        <x:v>Objective rows are updated with the latest owner-remediation retest. Automated Fail: 0. Blocked: 0. Twenty populated records remain Owner Review Required (15 prior subjective rows plus five OAR dispositions); owner acceptance is not claimed.</x:v>
+        <x:v>Final exact-HEAD owner-remediation-02 retest is recorded at b9814549911306cc46ce6db321e0e2f4c354c4ec. Automated Fail: 0. Blocked: 0. Existing 20 Owner Review Required records remain open (15 prior subjective rows plus five OAR dispositions); the six current owner defects are documented in the updated checklist. Owner acceptance is not claimed.</x:v>
       </x:c>
       <x:c r="C10" s="83"/>
       <x:c r="D10" s="54" t="str">
@@ -1354,7 +1354,7 @@
         <x:v>Candidate HEAD tested</x:v>
       </x:c>
       <x:c r="B11" s="83" t="str">
-        <x:v>03569c28644e40c39cd836b8e2559a652914d006</x:v>
+        <x:v>b9814549911306cc46ce6db321e0e2f4c354c4ec</x:v>
       </x:c>
       <x:c r="C11" s="83"/>
       <x:c r="D11" s="54" t="str">
@@ -1583,7 +1583,7 @@
         <x:v>Owner execution workflow</x:v>
       </x:c>
       <x:c r="B21" s="62" t="str">
-        <x:v>Objective retest failures are cleared at the tested implementation SHA above. Review only the remaining visual, editorial, tone, and environment judgments in the owner checklist; do not treat this execution set as owner acceptance or certification.</x:v>
+        <x:v>Objective retest failures are cleared at exact candidate b9814549911306cc46ce6db321e0e2f4c354c4ec. Review only the remaining visual, editorial, tone, and environment judgments in the owner checklist; do not treat this execution set as owner acceptance or certification. The current gate is owner re-review of DEF-OWNER-01 through DEF-OWNER-06 against this exact SHA.</x:v>
       </x:c>
       <x:c r="C21" s="62"/>
       <x:c r="D21" s="62"/>
@@ -1789,10 +1789,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -1839,10 +1839,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -1889,10 +1889,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -1939,10 +1939,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -1989,10 +1989,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -2039,10 +2039,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -2089,10 +2089,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -2139,10 +2139,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -2189,10 +2189,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -2239,10 +2239,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O14" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -2289,10 +2289,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O15" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -2339,10 +2339,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O16" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims.</x:v>
+        <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -2389,10 +2389,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O17" s="70" t="str">
-        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
+        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -2439,10 +2439,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O18" s="71" t="str">
-        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge readable composition, clipping, and visual comfort across the five supported viewports.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge readable composition, clipping, and visual comfort across the five supported viewports. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean. Owner must judge the visual/editorial feel of the representative result despite objective variation passing.</x:v>
       </x:c>
       <x:c r="P18" s="71" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2471,7 +2471,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0d23498b8ac4b4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re209faabd74b4846"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2632,10 +2632,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -2682,10 +2682,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -2732,10 +2732,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -2782,10 +2782,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -2832,10 +2832,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -2882,10 +2882,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -2932,10 +2932,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -2982,10 +2982,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -3032,10 +3032,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -3082,10 +3082,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O14" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -3132,10 +3132,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O15" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -3182,10 +3182,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O16" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -3232,10 +3232,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O17" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -3282,10 +3282,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O18" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -3332,10 +3332,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O19" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -3382,10 +3382,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O20" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -3432,10 +3432,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O21" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -3482,10 +3482,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O22" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P22" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="84" customHeight="1">
@@ -3532,10 +3532,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O23" s="70" t="str">
-        <x:v>Retest passed: None of these is mutually exclusive with every positive disclosure, and switching either direction clears the conflicting selections.</x:v>
+        <x:v>Retest passed: None of these is mutually exclusive with every positive disclosure, and switching either direction clears the conflicting selections. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P23" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -3582,10 +3582,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O24" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P24" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="84" customHeight="1">
@@ -3632,10 +3632,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O25" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P25" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="84" customHeight="1">
@@ -3682,10 +3682,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O26" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P26" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="84" customHeight="1">
@@ -3732,10 +3732,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O27" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P27" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="84" customHeight="1">
@@ -3782,10 +3782,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O28" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P28" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="84" customHeight="1">
@@ -3832,10 +3832,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O29" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P29" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="84" customHeight="1">
@@ -3882,10 +3882,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O30" s="70" t="str">
-        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented.</x:v>
+        <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P30" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="84" customHeight="1">
@@ -3932,10 +3932,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O31" s="70" t="str">
-        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the fallback-copy affordance and editorial naturalness after the exact success/blocked mechanics passed.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the fallback-copy affordance and editorial naturalness after the exact success/blocked mechanics passed. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements. Owner must judge the generated statement aloud for tone, rhythm, and conversational naturalness.</x:v>
       </x:c>
       <x:c r="P31" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; docs/qa/evidence/owner-remediation-01/console-log.txt; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; docs/qa/evidence/owner-remediation-01/console-log.txt; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="84" customHeight="1">
@@ -3982,10 +3982,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O32" s="70" t="str">
-        <x:v>Retest passed: the final step uses the named primary Build my pregame statement action, remains disabled until valid, preserves Back and multi-select, and reaches the result directly.</x:v>
+        <x:v>Retest passed: the final step uses the named primary Build my pregame statement action, remains disabled until valid, preserves Back and multi-select, and reaches the result directly. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P32" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/before-game-final-step-continue.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/before-game-final-step-continue.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="84" customHeight="1">
@@ -4032,10 +4032,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O33" s="71" t="str">
-        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge long-copy wrapping, result-card readability, and visual/editorial comfort.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge long-copy wrapping, result-card readability, and visual/editorial comfort. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements. Owner must judge the extreme disclosure statement for readability and practical table usability.</x:v>
       </x:c>
       <x:c r="P33" s="71" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4064,7 +4064,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R304adcc5348c4684"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01c5e893cad64a57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4225,10 +4225,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -4275,10 +4275,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -4325,10 +4325,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -4375,10 +4375,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -4425,10 +4425,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -4475,10 +4475,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -4525,10 +4525,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -4575,10 +4575,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs.</x:v>
+        <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -4625,10 +4625,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
+        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -4675,10 +4675,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O14" s="70" t="str">
-        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
+        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -4725,10 +4725,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O15" s="70" t="str">
-        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
+        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -4775,10 +4775,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O16" s="70" t="str">
-        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication.</x:v>
+        <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -4825,10 +4825,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O17" s="70" t="str">
-        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the thin-flow visual hierarchy and readability.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the thin-flow visual hierarchy and readability. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent. Owner must judge the six-moment result tone and the reordered neutral-sentence presentation.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -4875,10 +4875,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O18" s="71" t="str">
-        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
+        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P18" s="71" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4907,7 +4907,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf4d0028ec9b4993"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4e726581b07495e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5068,10 +5068,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -5118,10 +5118,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -5168,10 +5168,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -5218,10 +5218,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -5268,10 +5268,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -5318,10 +5318,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -5368,10 +5368,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -5418,10 +5418,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -5468,10 +5468,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -5518,10 +5518,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O14" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -5568,10 +5568,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O15" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -5618,10 +5618,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O16" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -5668,10 +5668,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O17" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -5718,10 +5718,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O18" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -5768,10 +5768,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O19" s="70" t="str">
-        <x:v>Retest passed through direct repository Puppeteer: native buttons activated with Enter and Space, lifecycle link activated with Enter, focus remained visible, and the final action/copy action were keyboard-operable without a focus trap.</x:v>
+        <x:v>Retest passed through direct repository Puppeteer: native buttons activated with Enter and Space, lifecycle link activated with Enter, focus remained visible, and the final action/copy action were keyboard-operable without a focus trap. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser keyboard trace; native button/link static inspection</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser keyboard trace; native button/link static inspection; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -5818,10 +5818,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O20" s="70" t="str">
-        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
+        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -5868,10 +5868,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O21" s="70" t="str">
-        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it.</x:v>
+        <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -5918,10 +5918,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O22" s="70" t="str">
-        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the visible focus ring, visual overlap, and settled scrolling.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the visible focus ring, visual overlap, and settled scrolling. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics. Owner must judge reduced-motion presentation and physical keyboard feel; native semantics and focus mechanics passed.</x:v>
       </x:c>
       <x:c r="P22" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="84" customHeight="1">
@@ -5968,10 +5968,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O23" s="70" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P23" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -6018,10 +6018,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O24" s="71" t="str">
-        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected.</x:v>
+        <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P24" s="71" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6050,7 +6050,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7214eb9fef844848"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8bdc2f66ff24b60"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6211,10 +6211,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -6261,10 +6261,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -6311,10 +6311,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -6361,10 +6361,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -6411,10 +6411,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -6461,10 +6461,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -6511,10 +6511,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -6561,10 +6561,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -6611,10 +6611,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -6661,10 +6661,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O14" s="70" t="str">
-        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge mobile hub visual balance and focus-ring visibility.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge mobile hub visual balance and focus-ring visibility. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks. Owner must judge desktop visual balance of the hub cards and Console preview density.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -6711,10 +6711,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O15" s="70" t="str">
-        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge focus-ring appearance and traversal feel.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge focus-ring appearance and traversal feel. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks. Owner must judge mobile visual balance, wrapping, and touch density.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -6761,10 +6761,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O16" s="70" t="str">
-        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge fallback feedback tone and lack of misleading persistence language.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge fallback feedback tone and lack of misleading persistence language. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks. Owner must judge existing After-the-Game visual/editorial continuity.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; docs/qa/evidence/owner-remediation-01/console-log.txt; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; docs/qa/evidence/owner-remediation-01/console-log.txt; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -6811,10 +6811,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O17" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -6861,10 +6861,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O18" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -6911,10 +6911,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O19" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -6961,10 +6961,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O20" s="70" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -7011,10 +7011,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O21" s="70" t="str">
-        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge reduced-motion settling and readability.</x:v>
+        <x:v>Retest objective portion passed at 2026-07-31. Owner must judge reduced-motion settling and readability. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks. Owner must judge existing Commander Console visual/interaction continuity.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -7061,10 +7061,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O22" s="71" t="str">
-        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites.</x:v>
+        <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P22" s="71" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7093,7 +7093,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a82cce515c741b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R419eedd8db6843fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7254,10 +7254,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O5" s="70" t="str">
-        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
+        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -7304,10 +7304,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O6" s="70" t="str">
-        <x:v>Retest passed exact visible-to-clipboard matching and truthful blocked feedback; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
+        <x:v>Retest passed exact visible-to-clipboard matching and truthful blocked feedback; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -7354,10 +7354,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O7" s="70" t="str">
-        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -7404,10 +7404,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O8" s="70" t="str">
-        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
+        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -7454,10 +7454,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O9" s="70" t="str">
-        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
+        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -7504,10 +7504,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O10" s="71" t="str">
-        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P10" s="71" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -7554,10 +7554,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O11" t="str">
-        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P11" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: git status/rev-parse; workbook artifact-tool inspect</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: git status/rev-parse; workbook artifact-tool inspect; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -7604,10 +7604,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O12" t="str">
-        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P12" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; command outputs</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; command outputs; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -7654,10 +7654,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O13" t="str">
-        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P13" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -7704,10 +7704,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O14" t="str">
-        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P14" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -7754,10 +7754,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O15" t="str">
-        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P15" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -7804,10 +7804,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O16" t="str">
-        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context.</x:v>
+        <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P16" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser history/keyboard trace; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser history/keyboard trace; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -7854,10 +7854,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O17" t="str">
-        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
+        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P17" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; browser console trace</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; browser console trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -7904,10 +7904,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O18" t="str">
-        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist.</x:v>
+        <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P18" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -7954,10 +7954,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O19" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P19" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; QA baseline commit 953a9052d2b056ed39051f11e247938fa60555d4</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; QA baseline commit 953a9052d2b056ed39051f11e247938fa60555d4; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -8004,10 +8004,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O20" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P20" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -8054,10 +8054,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O21" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P21" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -8104,10 +8104,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O22" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P22" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -8154,10 +8154,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O23" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P23" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -8204,10 +8204,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O24" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P24" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; docs/qa/evidence/retest-01/before-final-action-390x844.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; docs/qa/evidence/retest-01/before-final-action-390x844.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -8254,10 +8254,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O25" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P25" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -8304,10 +8304,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O26" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P26" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-01/retest-summary.json</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-01/retest-summary.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -8354,10 +8354,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O27" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P27" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; Previous retest: docs/qa/evidence/retest-01/retest-summary.json</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; Previous retest: docs/qa/evidence/retest-01/retest-summary.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -8404,10 +8404,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O28" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P28" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -8454,10 +8454,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O29" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P29" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -8504,10 +8504,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O30" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P30" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-review; npm.cmd run test:strategium-lifecycle</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-review; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -8554,10 +8554,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O31" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P31" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-final-action-390x844.png; docs/qa/evidence/retest-02/before-game-result-320x568.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-final-action-390x844.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -8604,10 +8604,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O32" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P32" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -8654,10 +8654,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O33" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P33" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:copy-boundaries; npm.cmd run test:route-metadata; npm.cmd run test:frontend-smoke; npm.cmd run test:parser; npm.cmd run test:browser-smoke; npm.cmd test</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:copy-boundaries; npm.cmd run test:route-metadata; npm.cmd run test:frontend-smoke; npm.cmd run test:parser; npm.cmd run test:browser-smoke; npm.cmd test; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -8704,10 +8704,10 @@
         <x:v>Automated Pass</x:v>
       </x:c>
       <x:c r="O34" t="str">
-        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status.</x:v>
+        <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P34" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-02/retest-summary.json</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-02/retest-summary.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -8754,10 +8754,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O35" t="str">
-        <x:v>OAR-01 remediated; owner re-review required.</x:v>
+        <x:v>OAR-01 remediated; owner re-review required. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P35" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -8804,10 +8804,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O36" t="str">
-        <x:v>OAR-02 remediated; owner re-review required.</x:v>
+        <x:v>OAR-02 remediated; owner re-review required. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P36" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -8854,10 +8854,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O37" t="str">
-        <x:v>OAR-03 remediated; owner re-review required.</x:v>
+        <x:v>OAR-03 remediated; owner re-review required. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P37" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -8904,10 +8904,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O38" t="str">
-        <x:v>OAR-04 remediated; owner re-review required.</x:v>
+        <x:v>OAR-04 remediated; owner re-review required. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P38" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -8954,10 +8954,10 @@
         <x:v>Owner Review Required</x:v>
       </x:c>
       <x:c r="O39" t="str">
-        <x:v>OAR-05 remediated; owner re-review required.</x:v>
+        <x:v>OAR-05 remediated; owner re-review required. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P39" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8989,7 +8989,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90f05ba0cfaf41ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9bfd6d524c34199"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
qa(strategium): record final copy and paths retest
</commit_message>
<xml_diff>
--- a/docs/qa/Strategium_Game_Lifecycle_Human_QA_Workbook.xlsx
+++ b/docs/qa/Strategium_Game_Lifecycle_Human_QA_Workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6ee11ef2981b4a5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finding a Table" sheetId="2" r:id="Re84f4b4f0d884a0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before the Game" sheetId="3" r:id="Rf46205a643a34ddc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="During the Game" sheetId="4" r:id="R6e1dc0e283a5497e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="5" r:id="R17d67ef50b684a42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation and Regression" sheetId="6" r:id="Rbff4c7a5113c4936"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human QA Log" sheetId="7" r:id="R9f5c3af32f614418"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4168e2509143449b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finding a Table" sheetId="2" r:id="Rcd8a496079a540ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before the Game" sheetId="3" r:id="R3d544945236a45db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="During the Game" sheetId="4" r:id="R508e0e6ae09d4673"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="5" r:id="R67aa37a156c54048"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation and Regression" sheetId="6" r:id="R5d1222245e45405e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human QA Log" sheetId="7" r:id="Rca376fb89d8a4c88"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1246,7 +1246,7 @@
         <x:v>Exact remediated candidate SHA</x:v>
       </x:c>
       <x:c r="B5" s="52" t="str">
-        <x:v>b9814549911306cc46ce6db321e0e2f4c354c4ec</x:v>
+        <x:v>99bd02481405e896780dc3067512eacac8cfa602</x:v>
       </x:c>
       <x:c r="C5" s="49"/>
       <x:c r="D5" s="53" t="str">
@@ -1335,7 +1335,7 @@
         <x:v>Execution status after automated retest</x:v>
       </x:c>
       <x:c r="B10" s="55" t="str">
-        <x:v>Final exact-HEAD owner-remediation-02 retest is recorded at b9814549911306cc46ce6db321e0e2f4c354c4ec. Automated Fail: 0. Blocked: 0. Existing 20 Owner Review Required records remain open (15 prior subjective rows plus five OAR dispositions); the six current owner defects are documented in the updated checklist. Owner acceptance is not claimed.</x:v>
+        <x:v>Final exact-HEAD three-defect owner-remediation retest is recorded at 99bd02481405e896780dc3067512eacac8cfa602. Automated Fail: 0. Blocked: 0. Existing 20 Owner Review Required records remain open; the two current owner defects are documented in the updated checklist. Owner acceptance is not claimed.</x:v>
       </x:c>
       <x:c r="C10" s="83"/>
       <x:c r="D10" s="54" t="str">
@@ -1354,7 +1354,7 @@
         <x:v>Candidate HEAD tested</x:v>
       </x:c>
       <x:c r="B11" s="83" t="str">
-        <x:v>b9814549911306cc46ce6db321e0e2f4c354c4ec</x:v>
+        <x:v>99bd02481405e896780dc3067512eacac8cfa602</x:v>
       </x:c>
       <x:c r="C11" s="83"/>
       <x:c r="D11" s="54" t="str">
@@ -1583,7 +1583,7 @@
         <x:v>Owner execution workflow</x:v>
       </x:c>
       <x:c r="B21" s="62" t="str">
-        <x:v>Objective retest failures are cleared at exact candidate b9814549911306cc46ce6db321e0e2f4c354c4ec. Review only the remaining visual, editorial, tone, and environment judgments in the owner checklist; do not treat this execution set as owner acceptance or certification. The current gate is owner re-review of DEF-OWNER-01 through DEF-OWNER-06 against this exact SHA.</x:v>
+        <x:v>Objective retest failures are cleared at exact candidate 99bd02481405e896780dc3067512eacac8cfa602. Review only the two current owner UX judgments in the owner checklist; do not treat this execution set as owner acceptance or certification. The current gate is owner re-review of the two Copy labels and centered Available Paths card against this exact SHA.</x:v>
       </x:c>
       <x:c r="C21" s="62"/>
       <x:c r="D21" s="62"/>
@@ -1792,7 +1792,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -1842,7 +1842,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -1892,7 +1892,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -1942,7 +1942,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -1992,7 +1992,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -2042,7 +2042,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -2092,7 +2092,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -2142,7 +2142,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -2192,7 +2192,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -2242,7 +2242,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -2292,7 +2292,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -2342,7 +2342,7 @@
         <x:v>Owner-remediation retest passed: all 1,200 combinations remained valid; the four-card result has the specific headline once, no Provisional compatibility read card, varied interpreted explanations/follow-ups/mismatch warnings, and no score, rating, certainty, or permanent player-label claims. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -2392,7 +2392,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -2442,7 +2442,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge readable composition, clipping, and visual comfort across the five supported viewports. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,200 deterministic combinations; the compatibility headline appears once, the Provisional card is absent, the four required cards remain, interpretation varies by selected signals, and safety boundaries remain clean. Owner must judge the visual/editorial feel of the representative result despite objective variation passing.</x:v>
       </x:c>
       <x:c r="P18" s="71" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/finding-a-table-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run test:route-metadata; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/finding-result-footer.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2471,7 +2471,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re209faabd74b4846"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbea9998740c74863"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2635,7 +2635,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -2685,7 +2685,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -2735,7 +2735,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -2785,7 +2785,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -2835,7 +2835,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -2885,7 +2885,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -2935,7 +2935,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -2985,7 +2985,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -3035,7 +3035,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -3085,7 +3085,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -3135,7 +3135,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -3185,7 +3185,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -3235,7 +3235,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -3285,7 +3285,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -3335,7 +3335,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -3385,7 +3385,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -3435,7 +3435,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -3485,7 +3485,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P22" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="84" customHeight="1">
@@ -3535,7 +3535,7 @@
         <x:v>Retest passed: None of these is mutually exclusive with every positive disclosure, and switching either direction clears the conflicting selections. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P23" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -3585,7 +3585,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P24" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="84" customHeight="1">
@@ -3635,7 +3635,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P25" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="84" customHeight="1">
@@ -3685,7 +3685,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P26" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="84" customHeight="1">
@@ -3735,7 +3735,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P27" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="84" customHeight="1">
@@ -3785,7 +3785,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P28" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="84" customHeight="1">
@@ -3835,7 +3835,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P29" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="84" customHeight="1">
@@ -3885,7 +3885,7 @@
         <x:v>Retest passed: the complete 1,935,360-output audit found zero semicolon-chain statements, malformed grammar cases, lost disclosures, unresolved IDs, duplicate clauses, or empty optional fragments; bracket, unsure, not-using, still-figuring-it-out, agreement, and disclosure partitions are represented. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P30" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="84" customHeight="1">
@@ -3935,7 +3935,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the fallback-copy affordance and editorial naturalness after the exact success/blocked mechanics passed. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements. Owner must judge the generated statement aloud for tone, rhythm, and conversational naturalness.</x:v>
       </x:c>
       <x:c r="P31" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; docs/qa/evidence/owner-remediation-01/console-log.txt; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; docs/qa/evidence/owner-remediation-01/console-log.txt; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="84" customHeight="1">
@@ -3985,7 +3985,7 @@
         <x:v>Retest passed: the final step uses the named primary Build my pregame statement action, remains disabled until valid, preserves Back and multi-select, and reaches the result directly. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements.</x:v>
       </x:c>
       <x:c r="P32" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/before-game-final-step-continue.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/before-game-final-step-continue.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="84" customHeight="1">
@@ -4035,7 +4035,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge long-copy wrapping, result-card readability, and visual/editorial comfort. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 1,935,360 combinations; maximum statement length 352/360 characters; zero lowercase openings, incorrect conjunctions, repeated conjunction chains, malformed disclosure lists, missing disclosures, unresolved IDs, duplicate clauses, semicolon chains, or over-limit statements. Owner must judge the extreme disclosure statement for readability and practical table usability.</x:v>
       </x:c>
       <x:c r="P33" s="71" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/before-game-result.png; docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/before-game-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/evidence/owner-remediation-02/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-02/before-step5-footer.png; docs/qa/evidence/owner-remediation-02/before-step6-before-selection.png; docs/qa/evidence/owner-remediation-02/before-step6-after-selection.png; npm.cmd run test:strategium-lifecycle; npm.cmd run lint:js; npm.cmd run lint:html. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; npm.cmd run test:copy-boundaries; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4064,7 +4064,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01c5e893cad64a57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a1db6035b254464"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4228,7 +4228,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -4278,7 +4278,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -4328,7 +4328,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -4378,7 +4378,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -4428,7 +4428,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -4478,7 +4478,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -4528,7 +4528,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -4578,7 +4578,7 @@
         <x:v>Retest passed: all six moments and all 48 moment/response pairs render the selected response label and response-specific guidance with zero fallback pairs. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -4628,7 +4628,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -4678,7 +4678,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -4728,7 +4728,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -4778,7 +4778,7 @@
         <x:v>Retest passed: all reachable During-the-Game output remained neutral and contained zero target, attack, removal, threat-score, player-rating, tactical, invented-ruling, objective-correctness, or table-politics advice; rules paths point to official lookup or human adjudication. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; npm.cmd run test:strategium-lifecycle; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -4828,7 +4828,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the thin-flow visual hierarchy and readability. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent. Owner must judge the six-moment result tone and the reordered neutral-sentence presentation.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -4878,7 +4878,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all 48 moment/response pairs; response labels and guidance are selected correctly, Available paths precedes the neutral sentence, copy equality is covered, and prohibited tactical/rating/ruling content remains absent.</x:v>
       </x:c>
       <x:c r="P18" s="71" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-02/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/during-result-reordered-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/evidence/owner-remediation-03/during-result-mobile.png; npm.cmd run test:strategium-lifecycle. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4907,7 +4907,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4e726581b07495e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9ca26d4ebdf477b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5071,7 +5071,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -5121,7 +5121,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -5171,7 +5171,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -5221,7 +5221,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -5271,7 +5271,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -5321,7 +5321,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -5371,7 +5371,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -5421,7 +5421,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -5471,7 +5471,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -5521,7 +5521,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -5571,7 +5571,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -5621,7 +5621,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -5671,7 +5671,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -5721,7 +5721,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -5771,7 +5771,7 @@
         <x:v>Retest passed through direct repository Puppeteer: native buttons activated with Enter and Space, lifecycle link activated with Enter, focus remained visible, and the final action/copy action were keyboard-operable without a focus trap. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser keyboard trace; native button/link static inspection; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser keyboard trace; native button/link static inspection; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -5821,7 +5821,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -5871,7 +5871,7 @@
         <x:v>Retest passed: invalid, incomplete, malformed, and extra state now shows the polite role=status recovery notice and lands on the nearest safe state; clean valid routes and ordinary history do not show it. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser URL trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -5921,7 +5921,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge the visible focus ring, visual overlap, and settled scrolling. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics. Owner must judge reduced-motion presentation and physical keyboard feel; native semantics and focus mechanics passed.</x:v>
       </x:c>
       <x:c r="P22" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="84" customHeight="1">
@@ -5971,7 +5971,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P23" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -6021,7 +6021,7 @@
         <x:v>Retest passed: initial load, selection, change, Continue, Back, result, reset, refresh, direct partial/complete load, hub return, Back/Forward, recovery, and valid-state persistence behaved as expected. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed initial load, selection/change, Continue, Back, result, reset, refresh, direct partial/complete state, hub return, browser history, recovery, focus, native keyboard semantics, and responsive mechanics.</x:v>
       </x:c>
       <x:c r="P24" s="71" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-lifecycle; browser history/recovery trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-02/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; npm.cmd run test:strategium-lifecycle; docs/qa/evidence/owner-remediation-03/direct-clean-review.png. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6050,7 +6050,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8bdc2f66ff24b60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64116f6740334316"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6214,7 +6214,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -6264,7 +6264,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -6314,7 +6314,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -6364,7 +6364,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -6414,7 +6414,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -6464,7 +6464,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P10" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -6514,7 +6514,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P11" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -6564,7 +6564,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P12" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -6614,7 +6614,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P13" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="84" customHeight="1">
@@ -6664,7 +6664,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge mobile hub visual balance and focus-ring visibility. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks. Owner must judge desktop visual balance of the hub cards and Console preview density.</x:v>
       </x:c>
       <x:c r="P14" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -6714,7 +6714,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge focus-ring appearance and traversal feel. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks. Owner must judge mobile visual balance, wrapping, and touch density.</x:v>
       </x:c>
       <x:c r="P15" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -6764,7 +6764,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge fallback feedback tone and lack of misleading persistence language. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks. Owner must judge existing After-the-Game visual/editorial continuity.</x:v>
       </x:c>
       <x:c r="P16" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; docs/qa/evidence/owner-remediation-01/console-log.txt; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; docs/qa/evidence/owner-remediation-01/console-log.txt; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: browser clipboard trace; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -6814,7 +6814,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P17" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -6864,7 +6864,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P18" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -6914,7 +6914,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P19" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -6964,7 +6964,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P20" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="84" customHeight="1">
@@ -7014,7 +7014,7 @@
         <x:v>Retest objective portion passed at 2026-07-31. Owner must judge reduced-motion settling and readability. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks. Owner must judge existing Commander Console visual/interaction continuity.</x:v>
       </x:c>
       <x:c r="P21" s="70" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; responsive browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -7064,7 +7064,7 @@
         <x:v>Owner-remediation retest passed: all four hub lifecycle links, direct hub-click After-the-Game entry, Commander Console previews, global navigation, canonical metadata, no stale selector labels, no dead ends, mobile overflow, and preserved review behavior were verified by the focused/regression suites. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest passed all four hub links, direct and hub-click After-the-Game entry, fresh-server route identity, stale-copy absence on reachable routes, global navigation, Console/review regression, metadata, smoke, and mobile overflow checks.</x:v>
       </x:c>
       <x:c r="P22" s="71" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/retest-summary.json; docs/qa/evidence/owner-remediation-01/browser-assertions.json; docs/qa/evidence/owner-remediation-01/copy-audit.json; docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:browser-smoke; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; First-run: npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata; browser trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/hub-desktop.png; docs/qa/evidence/owner-remediation-02/hub-mobile.png; docs/qa/evidence/owner-remediation-02/direct-clean-review.png; docs/qa/evidence/owner-remediation-02/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/hub-desktop.png; docs/qa/evidence/owner-remediation-03/hub-mobile.png; docs/qa/evidence/owner-remediation-03/direct-clean-review.png; docs/qa/evidence/owner-remediation-03/hub-click-review.png; npm.cmd run test:strategium-review; npm.cmd run test:browser-smoke; npm.cmd run test:route-metadata. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7093,7 +7093,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R419eedd8db6843fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cca055bddb44e39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7257,7 +7257,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P5" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -7307,7 +7307,7 @@
         <x:v>Retest passed exact visible-to-clipboard matching and truthful blocked feedback; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P6" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -7357,7 +7357,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P7" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -7407,7 +7407,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P8" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -7457,7 +7457,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P9" s="70" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; browser evidence; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -7507,7 +7507,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P10" s="71" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-game-lifecycle-mvp.md; npm.cmd run test:strategium-review; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -7557,7 +7557,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P11" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: git status/rev-parse; workbook artifact-tool inspect; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: git status/rev-parse; workbook artifact-tool inspect; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -7607,7 +7607,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P12" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; command outputs; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/during-response-pair-audit.json; command outputs; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -7657,7 +7657,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P13" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -7707,7 +7707,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P14" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/evaluator-audit.json; docs/qa/evidence/before-the-game-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -7757,7 +7757,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P15" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/during-response-pair-audit.json; docs/qa/evidence/during-the-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -7807,7 +7807,7 @@
         <x:v>Retest passed the objective portion; the original first-run evidence remains linked below as historical baseline context. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P16" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser history/keyboard trace; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/finding-a-table-invalid-recovery.png; browser history/keyboard trace; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -7857,7 +7857,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P17" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; browser console trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/strategium-hub-1440x900.png; docs/qa/evidence/during-game-initial-320x568-viewport-settled.png; browser console trace; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -7907,7 +7907,7 @@
         <x:v>Retest objective portion passed; Owner must complete the remaining subjective acceptance judgment listed in the checklist. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P18" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -7957,7 +7957,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P19" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; QA baseline commit 953a9052d2b056ed39051f11e247938fa60555d4; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; QA baseline commit 953a9052d2b056ed39051f11e247938fa60555d4; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -8007,7 +8007,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P20" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; First-run: docs/qa/evidence/; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -8057,7 +8057,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P21" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; npm.cmd run test:strategium-review; npm.cmd test; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -8107,7 +8107,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P22" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -8157,7 +8157,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P23" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/during-game-rules-result-1440x900.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -8207,7 +8207,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P24" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; docs/qa/evidence/retest-01/before-final-action-390x844.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/recovery-invalid-option-390x844.png; docs/qa/evidence/retest-01/before-final-action-390x844.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -8257,7 +8257,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P25" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-01/retest-summary.json; docs/qa/evidence/retest-01/hub-1440x900.png; docs/qa/evidence/retest-01/before-game-result-320x568.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -8307,7 +8307,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P26" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-01/retest-summary.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-01/retest-summary.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -8357,7 +8357,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P27" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; Previous retest: docs/qa/evidence/retest-01/retest-summary.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; Previous retest: docs/qa/evidence/retest-01/retest-summary.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -8407,7 +8407,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P28" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -8457,7 +8457,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P29" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -8507,7 +8507,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P30" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-review; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run test:strategium-review; npm.cmd run test:strategium-lifecycle; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -8557,7 +8557,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P31" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-final-action-390x844.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/before-final-action-390x844.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -8607,7 +8607,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P32" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; docs/qa/evidence/retest-02/hub-1440x900.png; docs/qa/evidence/retest-02/before-game-result-320x568.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -8657,7 +8657,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P33" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:copy-boundaries; npm.cmd run test:route-metadata; npm.cmd run test:frontend-smoke; npm.cmd run test:parser; npm.cmd run test:browser-smoke; npm.cmd test; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/evidence/retest-02/retest-summary.json; npm.cmd run lint:js; npm.cmd run lint:html; npm.cmd run test:copy-boundaries; npm.cmd run test:route-metadata; npm.cmd run test:frontend-smoke; npm.cmd run test:parser; npm.cmd run test:browser-smoke; npm.cmd test; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -8707,7 +8707,7 @@
         <x:v>Retest metadata remains preserved; see the new retest log records for exact identity, commands, and current status. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P34" t="str">
-        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-02/retest-summary.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>Retest: docs/qa/evidence/owner-remediation-01/retest-summary.json; First-run: Retest: docs/qa/evidence/retest-02/retest-summary.json; First-run: docs/qa/strategium-lifecycle-owner-acceptance-checklist.md; docs/qa/evidence/retest-02/retest-summary.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -8757,7 +8757,7 @@
         <x:v>OAR-01 remediated; owner re-review required. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P35" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/hub-desktop.png; docs/qa/evidence/owner-remediation-01/hub-mobile.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -8807,7 +8807,7 @@
         <x:v>OAR-02 remediated; owner re-review required. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P36" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/finding-a-table-result.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -8857,7 +8857,7 @@
         <x:v>OAR-03 remediated; owner re-review required. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P37" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/before-game-bracket-step.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -8907,7 +8907,7 @@
         <x:v>OAR-04 remediated; owner re-review required. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P38" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/before-game-step-5-action-footer.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-before-selection.png; docs/qa/evidence/owner-remediation-01/before-game-step-6-action-footer-after-selection.png; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -8957,7 +8957,7 @@
         <x:v>OAR-05 remediated; owner re-review required. Latest exact-HEAD owner-remediation-02 retest @ b9814549911306cc46ce6db321e0e2f4c354c4ec: Final exact-HEAD retest record: rejected candidate 52554cc4e6572e85301b89884b7513c23302ad82; tested implementation/final candidate b9814549911306cc46ce6db321e0e2f4c354c4ec; Automated Fail 0; Blocked 0; owner acceptance not claimed.</x:v>
       </x:c>
       <x:c r="P39" t="str">
-        <x:v>docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
+        <x:v>docs/qa/evidence/owner-remediation-01/after-game-hub-entry.png; docs/qa/evidence/owner-remediation-01/browser-assertions.json; Latest evidence @ b9814549911306cc46ce6db321e0e2f4c354c4ec: docs/qa/evidence/owner-remediation-02/browser-assertions.json; docs/qa/evidence/owner-remediation-02/before-game-copy-audit.json; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.; Latest evidence @ 48e4a2270c66fb9e417e2c5f4c2022619e4ceff2: docs/qa/evidence/owner-remediation-03/browser-assertions.json; docs/qa/evidence/owner-remediation-03/before-result-rich-copy.png; docs/qa/evidence/owner-remediation-03/during-result-copy-success.png; docs/qa/strategium-game-lifecycle-mvp.md; docs/qa/strategium-lifecycle-owner-acceptance-checklist.md. Historical baseline and prior retest references are preserved in the existing workbook text and evidence directories.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8989,7 +8989,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9bfd6d524c34199"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10a191cb0dce41cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>